<commit_message>
Segundo Parcial 7 noviembre noche
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -8003,7 +8003,7 @@
         <v>15.79</v>
       </c>
       <c r="I4" s="2">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -8376,16 +8376,16 @@
         <v>45</v>
       </c>
       <c r="E15">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G15" s="1">
-        <v>84.44</v>
+        <v>86.67</v>
       </c>
       <c r="H15" s="1">
-        <v>13.33</v>
+        <v>11.11</v>
       </c>
       <c r="I15" s="2">
         <v>6.8</v>
@@ -9020,16 +9020,19 @@
         <v>27</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F34">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="G34" s="1">
-        <v>0</v>
+        <v>96.3</v>
       </c>
       <c r="H34" s="1">
-        <v>100</v>
+        <v>3.7</v>
+      </c>
+      <c r="I34" s="2">
+        <v>8.199999999999999</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -9052,16 +9055,19 @@
         <v>21</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F35">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="G35" s="1">
-        <v>0</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="H35" s="1">
-        <v>100</v>
+        <v>14.29</v>
+      </c>
+      <c r="I35" s="2">
+        <v>8.1</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -9084,16 +9090,19 @@
         <v>26</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F36">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G36" s="1">
-        <v>0</v>
+        <v>61.54</v>
       </c>
       <c r="H36" s="1">
-        <v>100</v>
+        <v>38.46</v>
+      </c>
+      <c r="I36" s="2">
+        <v>6.1</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -9151,16 +9160,19 @@
         <v>19</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F38">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G38" s="1">
-        <v>0</v>
+        <v>57.89</v>
       </c>
       <c r="H38" s="1">
-        <v>73.68000000000001</v>
+        <v>15.79</v>
+      </c>
+      <c r="I38" s="2">
+        <v>7.7</v>
       </c>
       <c r="J38">
         <v>5</v>
@@ -9183,16 +9195,19 @@
         <v>34</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F39">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="G39" s="1">
-        <v>0</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="H39" s="1">
-        <v>82.34999999999999</v>
+        <v>17.65</v>
+      </c>
+      <c r="I39" s="2">
+        <v>7.4</v>
       </c>
       <c r="J39">
         <v>6</v>
@@ -9460,16 +9475,19 @@
         <v>44</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="F47">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="G47" s="1">
-        <v>0</v>
+        <v>95.45</v>
       </c>
       <c r="H47" s="1">
-        <v>100</v>
+        <v>4.55</v>
+      </c>
+      <c r="I47" s="2">
+        <v>8.5</v>
       </c>
       <c r="J47">
         <v>0</v>
@@ -9699,16 +9717,19 @@
         <v>34</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F54">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1">
-        <v>0</v>
+        <v>94.12</v>
       </c>
       <c r="H54" s="1">
-        <v>100</v>
+        <v>5.88</v>
+      </c>
+      <c r="I54" s="2">
+        <v>8.1</v>
       </c>
       <c r="J54">
         <v>0</v>
@@ -9731,16 +9752,19 @@
         <v>30</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F55">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="G55" s="1">
-        <v>0</v>
+        <v>86.67</v>
       </c>
       <c r="H55" s="1">
-        <v>100</v>
+        <v>13.33</v>
+      </c>
+      <c r="I55" s="2">
+        <v>7.6</v>
       </c>
       <c r="J55">
         <v>0</v>
@@ -9763,16 +9787,19 @@
         <v>40</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F56">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="G56" s="1">
-        <v>0</v>
+        <v>87.5</v>
       </c>
       <c r="H56" s="1">
-        <v>100</v>
+        <v>12.5</v>
+      </c>
+      <c r="I56" s="2">
+        <v>7.9</v>
       </c>
       <c r="J56">
         <v>0</v>
@@ -9795,16 +9822,19 @@
         <v>44</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="F57">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="G57" s="1">
-        <v>0</v>
+        <v>95.45</v>
       </c>
       <c r="H57" s="1">
-        <v>100</v>
+        <v>4.55</v>
+      </c>
+      <c r="I57" s="2">
+        <v>8.800000000000001</v>
       </c>
       <c r="J57">
         <v>0</v>
@@ -9827,16 +9857,19 @@
         <v>43</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F58">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="G58" s="1">
-        <v>0</v>
+        <v>86.05</v>
       </c>
       <c r="H58" s="1">
-        <v>100</v>
+        <v>13.95</v>
+      </c>
+      <c r="I58" s="2">
+        <v>8.199999999999999</v>
       </c>
       <c r="J58">
         <v>0</v>
@@ -9859,16 +9892,19 @@
         <v>43</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F59">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="G59" s="1">
-        <v>0</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="H59" s="1">
-        <v>100</v>
+        <v>20.93</v>
+      </c>
+      <c r="I59" s="2">
+        <v>7.8</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -10066,16 +10102,19 @@
         <v>40</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F65">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G65" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H65" s="1">
-        <v>100</v>
+        <v>20</v>
+      </c>
+      <c r="I65" s="2">
+        <v>6.3</v>
       </c>
       <c r="J65">
         <v>0</v>
@@ -10098,16 +10137,19 @@
         <v>44</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F66">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="G66" s="1">
-        <v>0</v>
+        <v>84.09</v>
       </c>
       <c r="H66" s="1">
-        <v>100</v>
+        <v>15.91</v>
+      </c>
+      <c r="I66" s="2">
+        <v>7.2</v>
       </c>
       <c r="J66">
         <v>0</v>
@@ -10130,16 +10172,19 @@
         <v>43</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F67">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="G67" s="1">
-        <v>0</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H67" s="1">
-        <v>100</v>
+        <v>23.26</v>
+      </c>
+      <c r="I67" s="2">
+        <v>6.7</v>
       </c>
       <c r="J67">
         <v>0</v>
@@ -10162,16 +10207,19 @@
         <v>43</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F68">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="G68" s="1">
-        <v>0</v>
+        <v>74.42</v>
       </c>
       <c r="H68" s="1">
-        <v>97.67</v>
+        <v>23.26</v>
+      </c>
+      <c r="I68" s="2">
+        <v>6.4</v>
       </c>
       <c r="J68">
         <v>1</v>
@@ -10194,16 +10242,19 @@
         <v>34</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F69">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G69" s="1">
-        <v>0</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="H69" s="1">
-        <v>97.06</v>
+        <v>32.35</v>
+      </c>
+      <c r="I69" s="2">
+        <v>6.7</v>
       </c>
       <c r="J69">
         <v>1</v>
@@ -10226,16 +10277,19 @@
         <v>34</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F70">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="G70" s="1">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H70" s="1">
-        <v>88.23999999999999</v>
+        <v>38.24</v>
+      </c>
+      <c r="I70" s="2">
+        <v>8.5</v>
       </c>
       <c r="J70">
         <v>4</v>
@@ -10258,16 +10312,19 @@
         <v>38</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F71">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="G71" s="1">
-        <v>0</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="H71" s="1">
-        <v>89.47</v>
+        <v>15.79</v>
+      </c>
+      <c r="I71" s="2">
+        <v>8.1</v>
       </c>
       <c r="J71">
         <v>4</v>
@@ -10290,16 +10347,19 @@
         <v>32</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F72">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="G72" s="1">
-        <v>0</v>
+        <v>81.25</v>
       </c>
       <c r="H72" s="1">
-        <v>93.75</v>
+        <v>12.5</v>
+      </c>
+      <c r="I72" s="2">
+        <v>8.9</v>
       </c>
       <c r="J72">
         <v>2</v>
@@ -10322,16 +10382,19 @@
         <v>26</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F73">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G73" s="1">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H73" s="1">
-        <v>65.38</v>
+        <v>15.38</v>
+      </c>
+      <c r="I73" s="2">
+        <v>7.7</v>
       </c>
       <c r="J73">
         <v>9</v>
@@ -10354,16 +10417,19 @@
         <v>33</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F74">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="G74" s="1">
-        <v>0</v>
+        <v>72.73</v>
       </c>
       <c r="H74" s="1">
-        <v>81.81999999999999</v>
+        <v>9.09</v>
+      </c>
+      <c r="I74" s="2">
+        <v>9.5</v>
       </c>
       <c r="J74">
         <v>6</v>
@@ -10931,16 +10997,19 @@
         <v>36</v>
       </c>
       <c r="E91">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F91">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="G91" s="1">
-        <v>0</v>
+        <v>83.33</v>
       </c>
       <c r="H91" s="1">
-        <v>86.11</v>
+        <v>2.78</v>
+      </c>
+      <c r="I91" s="2">
+        <v>7.3</v>
       </c>
       <c r="J91">
         <v>5</v>
@@ -10998,16 +11067,19 @@
         <v>30</v>
       </c>
       <c r="E93">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F93">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G93" s="1">
-        <v>0</v>
+        <v>83.33</v>
       </c>
       <c r="H93" s="1">
-        <v>100</v>
+        <v>16.67</v>
+      </c>
+      <c r="I93" s="2">
+        <v>7</v>
       </c>
       <c r="J93">
         <v>0</v>
@@ -11030,16 +11102,19 @@
         <v>32</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F94">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="G94" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H94" s="1">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="I94" s="2">
+        <v>9.5</v>
       </c>
       <c r="J94">
         <v>0</v>
@@ -11097,16 +11172,19 @@
         <v>18</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F96">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G96" s="1">
-        <v>0</v>
+        <v>88.89</v>
       </c>
       <c r="H96" s="1">
-        <v>100</v>
+        <v>11.11</v>
+      </c>
+      <c r="I96" s="2">
+        <v>7.4</v>
       </c>
       <c r="J96">
         <v>0</v>
@@ -11129,16 +11207,19 @@
         <v>41</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F97">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="G97" s="1">
-        <v>0</v>
+        <v>87.8</v>
       </c>
       <c r="H97" s="1">
-        <v>87.8</v>
+        <v>0</v>
+      </c>
+      <c r="I97" s="2">
+        <v>9.300000000000001</v>
       </c>
       <c r="J97">
         <v>5</v>
@@ -12208,16 +12289,19 @@
         <v>34</v>
       </c>
       <c r="E128">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F128">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="G128" s="1">
-        <v>0</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H128" s="1">
-        <v>100</v>
+        <v>32.35</v>
+      </c>
+      <c r="I128" s="2">
+        <v>6.4</v>
       </c>
       <c r="J128">
         <v>0</v>
@@ -12240,19 +12324,19 @@
         <v>30</v>
       </c>
       <c r="E129">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F129">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G129" s="1">
-        <v>56.67</v>
+        <v>60</v>
       </c>
       <c r="H129" s="1">
-        <v>43.33</v>
+        <v>40</v>
       </c>
       <c r="I129" s="2">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="J129">
         <v>0</v>
@@ -12287,7 +12371,7 @@
         <v>35</v>
       </c>
       <c r="I130" s="2">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -12322,7 +12406,7 @@
         <v>13.64</v>
       </c>
       <c r="I131" s="2">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="J131">
         <v>0</v>
@@ -12345,16 +12429,19 @@
         <v>43</v>
       </c>
       <c r="E132">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F132">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="G132" s="1">
-        <v>0</v>
+        <v>74.42</v>
       </c>
       <c r="H132" s="1">
-        <v>100</v>
+        <v>25.58</v>
+      </c>
+      <c r="I132" s="2">
+        <v>7.1</v>
       </c>
       <c r="J132">
         <v>0</v>
@@ -12377,16 +12464,19 @@
         <v>43</v>
       </c>
       <c r="E133">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F133">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="G133" s="1">
-        <v>0</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="H133" s="1">
-        <v>100</v>
+        <v>20.93</v>
+      </c>
+      <c r="I133" s="2">
+        <v>7</v>
       </c>
       <c r="J133">
         <v>0</v>
@@ -12409,16 +12499,16 @@
         <v>27</v>
       </c>
       <c r="E134">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F134">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G134" s="1">
-        <v>88.89</v>
+        <v>100</v>
       </c>
       <c r="H134" s="1">
-        <v>11.11</v>
+        <v>0</v>
       </c>
       <c r="I134" s="2">
         <v>8</v>
@@ -12444,16 +12534,19 @@
         <v>44</v>
       </c>
       <c r="E135">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F135">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="G135" s="1">
-        <v>0</v>
+        <v>79.55</v>
       </c>
       <c r="H135" s="1">
-        <v>100</v>
+        <v>20.45</v>
+      </c>
+      <c r="I135" s="2">
+        <v>7.1</v>
       </c>
       <c r="J135">
         <v>0</v>
@@ -13103,7 +13196,7 @@
         <v>3.13</v>
       </c>
       <c r="I154" s="2">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J154">
         <v>0</v>
@@ -13686,16 +13779,19 @@
         <v>21</v>
       </c>
       <c r="E171">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F171">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G171" s="1">
-        <v>0</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H171" s="1">
-        <v>100</v>
+        <v>4.76</v>
+      </c>
+      <c r="I171" s="2">
+        <v>8</v>
       </c>
       <c r="J171">
         <v>0</v>
@@ -13718,16 +13814,19 @@
         <v>39</v>
       </c>
       <c r="E172">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F172">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="G172" s="1">
-        <v>0</v>
+        <v>51.28</v>
       </c>
       <c r="H172" s="1">
-        <v>56.41</v>
+        <v>5.13</v>
+      </c>
+      <c r="I172" s="2">
+        <v>7.8</v>
       </c>
       <c r="J172">
         <v>17</v>
@@ -13995,16 +14094,19 @@
         <v>30</v>
       </c>
       <c r="E180">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F180">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G180" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H180" s="1">
-        <v>100</v>
+        <v>20</v>
+      </c>
+      <c r="I180" s="2">
+        <v>7.9</v>
       </c>
       <c r="J180">
         <v>0</v>
@@ -14347,16 +14449,19 @@
         <v>26</v>
       </c>
       <c r="E191">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F191">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="G191" s="1">
-        <v>0</v>
+        <v>61.54</v>
       </c>
       <c r="H191" s="1">
-        <v>84.62</v>
+        <v>23.08</v>
+      </c>
+      <c r="I191" s="2">
+        <v>6.8</v>
       </c>
       <c r="J191">
         <v>4</v>
@@ -14379,16 +14484,19 @@
         <v>15</v>
       </c>
       <c r="E192">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F192">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G192" s="1">
-        <v>0</v>
+        <v>46.67</v>
       </c>
       <c r="H192" s="1">
-        <v>100</v>
+        <v>53.33</v>
+      </c>
+      <c r="I192" s="2">
+        <v>6.1</v>
       </c>
       <c r="J192">
         <v>0</v>
@@ -14691,19 +14799,19 @@
         <v>45</v>
       </c>
       <c r="E201">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F201">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G201" s="1">
-        <v>80</v>
+        <v>86.67</v>
       </c>
       <c r="H201" s="1">
-        <v>20</v>
+        <v>13.33</v>
       </c>
       <c r="I201" s="2">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="J201">
         <v>0</v>
@@ -15268,16 +15376,16 @@
         <v>45</v>
       </c>
       <c r="E15">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="1">
-        <v>88.89</v>
+        <v>86.67</v>
       </c>
       <c r="H15" s="1">
-        <v>8.890000000000001</v>
+        <v>11.11</v>
       </c>
       <c r="I15" s="2">
         <v>7.4</v>
@@ -15933,16 +16041,16 @@
         <v>27</v>
       </c>
       <c r="E34">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="1">
-        <v>100</v>
+        <v>96.3</v>
       </c>
       <c r="H34" s="1">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="I34" s="2">
         <v>8.6</v>
@@ -15968,19 +16076,19 @@
         <v>21</v>
       </c>
       <c r="E35">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" s="1">
-        <v>90.48</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="H35" s="1">
-        <v>9.52</v>
+        <v>14.29</v>
       </c>
       <c r="I35" s="2">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -16003,19 +16111,19 @@
         <v>26</v>
       </c>
       <c r="E36">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F36">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G36" s="1">
-        <v>80.77</v>
+        <v>61.54</v>
       </c>
       <c r="H36" s="1">
-        <v>19.23</v>
+        <v>38.46</v>
       </c>
       <c r="I36" s="2">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -16073,19 +16181,19 @@
         <v>19</v>
       </c>
       <c r="E38">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G38" s="1">
-        <v>52.63</v>
+        <v>57.89</v>
       </c>
       <c r="H38" s="1">
-        <v>21.05</v>
+        <v>15.79</v>
       </c>
       <c r="I38" s="2">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="J38">
         <v>5</v>
@@ -16108,19 +16216,19 @@
         <v>34</v>
       </c>
       <c r="E39">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F39">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G39" s="1">
-        <v>50</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H39" s="1">
-        <v>32.35</v>
+        <v>14.71</v>
       </c>
       <c r="I39" s="2">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J39">
         <v>6</v>
@@ -16633,19 +16741,19 @@
         <v>34</v>
       </c>
       <c r="E54">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F54">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1">
-        <v>88.23999999999999</v>
+        <v>94.12</v>
       </c>
       <c r="H54" s="1">
-        <v>11.76</v>
+        <v>5.88</v>
       </c>
       <c r="I54" s="2">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="J54">
         <v>0</v>
@@ -16680,7 +16788,7 @@
         <v>13.33</v>
       </c>
       <c r="I55" s="2">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="J55">
         <v>0</v>
@@ -16703,19 +16811,19 @@
         <v>40</v>
       </c>
       <c r="E56">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G56" s="1">
-        <v>90</v>
+        <v>87.5</v>
       </c>
       <c r="H56" s="1">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="I56" s="2">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="J56">
         <v>0</v>
@@ -16750,7 +16858,7 @@
         <v>4.55</v>
       </c>
       <c r="I57" s="2">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="J57">
         <v>0</v>
@@ -16785,7 +16893,7 @@
         <v>13.95</v>
       </c>
       <c r="I58" s="2">
-        <v>7.1</v>
+        <v>7.8</v>
       </c>
       <c r="J58">
         <v>0</v>
@@ -16808,19 +16916,19 @@
         <v>43</v>
       </c>
       <c r="E59">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F59">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G59" s="1">
-        <v>83.72</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="H59" s="1">
-        <v>16.28</v>
+        <v>20.93</v>
       </c>
       <c r="I59" s="2">
-        <v>7</v>
+        <v>7.6</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -17018,19 +17126,19 @@
         <v>40</v>
       </c>
       <c r="E65">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F65">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G65" s="1">
-        <v>82.5</v>
+        <v>80</v>
       </c>
       <c r="H65" s="1">
-        <v>17.5</v>
+        <v>20</v>
       </c>
       <c r="I65" s="2">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="J65">
         <v>0</v>
@@ -17065,7 +17173,7 @@
         <v>15.91</v>
       </c>
       <c r="I66" s="2">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="J66">
         <v>0</v>
@@ -17088,19 +17196,19 @@
         <v>43</v>
       </c>
       <c r="E67">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F67">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G67" s="1">
-        <v>79.06999999999999</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H67" s="1">
-        <v>20.93</v>
+        <v>23.26</v>
       </c>
       <c r="I67" s="2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J67">
         <v>0</v>
@@ -17135,7 +17243,7 @@
         <v>23.26</v>
       </c>
       <c r="I68" s="2">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="J68">
         <v>1</v>
@@ -17158,19 +17266,19 @@
         <v>34</v>
       </c>
       <c r="E69">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F69">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G69" s="1">
-        <v>70.59</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="H69" s="1">
-        <v>26.47</v>
+        <v>32.35</v>
       </c>
       <c r="I69" s="2">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="J69">
         <v>1</v>
@@ -17205,7 +17313,7 @@
         <v>2.94</v>
       </c>
       <c r="I70" s="2">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="J70">
         <v>4</v>
@@ -17263,19 +17371,19 @@
         <v>32</v>
       </c>
       <c r="E72">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G72" s="1">
-        <v>90.63</v>
+        <v>93.75</v>
       </c>
       <c r="H72" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
       <c r="I72" s="2">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J72">
         <v>2</v>
@@ -17345,7 +17453,7 @@
         <v>0</v>
       </c>
       <c r="I74" s="2">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J74">
         <v>6</v>
@@ -17928,19 +18036,19 @@
         <v>36</v>
       </c>
       <c r="E91">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" s="1">
-        <v>86.11</v>
+        <v>83.33</v>
       </c>
       <c r="H91" s="1">
-        <v>0</v>
+        <v>2.78</v>
       </c>
       <c r="I91" s="2">
-        <v>7</v>
+        <v>7.4</v>
       </c>
       <c r="J91">
         <v>5</v>
@@ -17998,19 +18106,19 @@
         <v>30</v>
       </c>
       <c r="E93">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F93">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G93" s="1">
-        <v>80</v>
+        <v>83.33</v>
       </c>
       <c r="H93" s="1">
-        <v>20</v>
+        <v>16.67</v>
       </c>
       <c r="I93" s="2">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
       <c r="J93">
         <v>0</v>
@@ -18033,19 +18141,19 @@
         <v>32</v>
       </c>
       <c r="E94">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F94">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G94" s="1">
-        <v>78.13</v>
+        <v>100</v>
       </c>
       <c r="H94" s="1">
-        <v>21.88</v>
+        <v>0</v>
       </c>
       <c r="I94" s="2">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J94">
         <v>0</v>
@@ -18103,19 +18211,19 @@
         <v>18</v>
       </c>
       <c r="E96">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F96">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G96" s="1">
-        <v>83.33</v>
+        <v>88.89</v>
       </c>
       <c r="H96" s="1">
-        <v>16.67</v>
+        <v>11.11</v>
       </c>
       <c r="I96" s="2">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="J96">
         <v>0</v>
@@ -18150,7 +18258,7 @@
         <v>0</v>
       </c>
       <c r="I97" s="2">
-        <v>8.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J97">
         <v>5</v>
@@ -19223,19 +19331,19 @@
         <v>34</v>
       </c>
       <c r="E128">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F128">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G128" s="1">
-        <v>73.53</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H128" s="1">
-        <v>26.47</v>
+        <v>32.35</v>
       </c>
       <c r="I128" s="2">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="J128">
         <v>0</v>
@@ -19293,19 +19401,19 @@
         <v>40</v>
       </c>
       <c r="E130">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F130">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G130" s="1">
-        <v>67.5</v>
+        <v>65</v>
       </c>
       <c r="H130" s="1">
-        <v>32.5</v>
+        <v>35</v>
       </c>
       <c r="I130" s="2">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -19363,19 +19471,19 @@
         <v>43</v>
       </c>
       <c r="E132">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F132">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G132" s="1">
-        <v>81.40000000000001</v>
+        <v>74.42</v>
       </c>
       <c r="H132" s="1">
-        <v>18.6</v>
+        <v>25.58</v>
       </c>
       <c r="I132" s="2">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="J132">
         <v>0</v>
@@ -19398,19 +19506,19 @@
         <v>43</v>
       </c>
       <c r="E133">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F133">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G133" s="1">
-        <v>81.40000000000001</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="H133" s="1">
-        <v>18.6</v>
+        <v>20.93</v>
       </c>
       <c r="I133" s="2">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="J133">
         <v>0</v>
@@ -19468,19 +19576,19 @@
         <v>44</v>
       </c>
       <c r="E135">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F135">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G135" s="1">
-        <v>70.45</v>
+        <v>81.81999999999999</v>
       </c>
       <c r="H135" s="1">
-        <v>29.55</v>
+        <v>18.18</v>
       </c>
       <c r="I135" s="2">
-        <v>6.3</v>
+        <v>6.8</v>
       </c>
       <c r="J135">
         <v>0</v>
@@ -20133,16 +20241,16 @@
         <v>32</v>
       </c>
       <c r="E154">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F154">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G154" s="1">
-        <v>100</v>
+        <v>96.88</v>
       </c>
       <c r="H154" s="1">
-        <v>0</v>
+        <v>3.13</v>
       </c>
       <c r="I154" s="2">
         <v>8.5</v>
@@ -20728,19 +20836,19 @@
         <v>21</v>
       </c>
       <c r="E171">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F171">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G171" s="1">
-        <v>90.48</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H171" s="1">
-        <v>9.52</v>
+        <v>4.76</v>
       </c>
       <c r="I171" s="2">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="J171">
         <v>0</v>
@@ -20763,19 +20871,19 @@
         <v>39</v>
       </c>
       <c r="E172">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F172">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G172" s="1">
-        <v>56.41</v>
+        <v>51.28</v>
       </c>
       <c r="H172" s="1">
-        <v>0</v>
+        <v>5.13</v>
       </c>
       <c r="I172" s="2">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="J172">
         <v>17</v>
@@ -21043,19 +21151,19 @@
         <v>30</v>
       </c>
       <c r="E180">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F180">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G180" s="1">
-        <v>76.67</v>
+        <v>86.67</v>
       </c>
       <c r="H180" s="1">
-        <v>23.33</v>
+        <v>13.33</v>
       </c>
       <c r="I180" s="2">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="J180">
         <v>0</v>
@@ -21428,19 +21536,19 @@
         <v>26</v>
       </c>
       <c r="E191">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F191">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G191" s="1">
-        <v>84.62</v>
+        <v>61.54</v>
       </c>
       <c r="H191" s="1">
-        <v>0</v>
+        <v>23.08</v>
       </c>
       <c r="I191" s="2">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="J191">
         <v>4</v>
@@ -21475,7 +21583,7 @@
         <v>53.33</v>
       </c>
       <c r="I192" s="2">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="J192">
         <v>0</v>
@@ -21778,16 +21886,16 @@
         <v>45</v>
       </c>
       <c r="E201">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F201">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G201" s="1">
-        <v>88.89</v>
+        <v>86.67</v>
       </c>
       <c r="H201" s="1">
-        <v>11.11</v>
+        <v>13.33</v>
       </c>
       <c r="I201" s="2">
         <v>7.4</v>

</xml_diff>

<commit_message>
Segundo Parcial 12 noviembre
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -1394,25 +1394,25 @@
         <v>38</v>
       </c>
       <c r="E18">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G18" s="1">
-        <v>89.47</v>
+        <v>92.11</v>
       </c>
       <c r="H18" s="1">
-        <v>0</v>
+        <v>7.89</v>
       </c>
       <c r="I18" s="2">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2062,22 +2062,22 @@
         <v>13</v>
       </c>
       <c r="F37">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G37" s="1">
         <v>50</v>
       </c>
       <c r="H37" s="1">
-        <v>46.15</v>
+        <v>50</v>
       </c>
       <c r="I37" s="2">
         <v>6.2</v>
       </c>
       <c r="J37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="1">
-        <v>3.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2094,25 +2094,25 @@
         <v>19</v>
       </c>
       <c r="E38">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G38" s="1">
-        <v>52.63</v>
+        <v>57.89</v>
       </c>
       <c r="H38" s="1">
-        <v>21.05</v>
+        <v>42.11</v>
       </c>
       <c r="I38" s="2">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="J38">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K38" s="1">
-        <v>26.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2132,22 +2132,22 @@
         <v>17</v>
       </c>
       <c r="F39">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G39" s="1">
         <v>50</v>
       </c>
       <c r="H39" s="1">
-        <v>32.35</v>
+        <v>50</v>
       </c>
       <c r="I39" s="2">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K39" s="1">
-        <v>17.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2237,22 +2237,22 @@
         <v>34</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" s="1">
         <v>97.14</v>
       </c>
       <c r="H42" s="1">
-        <v>0</v>
+        <v>2.86</v>
       </c>
       <c r="I42" s="2">
         <v>7.9</v>
       </c>
       <c r="J42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" s="1">
-        <v>2.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2269,25 +2269,25 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="1">
-        <v>52.38</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H43" s="1">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="I43" s="2">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="J43">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K43" s="1">
-        <v>47.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2304,25 +2304,25 @@
         <v>37</v>
       </c>
       <c r="E44">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G44" s="1">
-        <v>67.56999999999999</v>
+        <v>81.08</v>
       </c>
       <c r="H44" s="1">
-        <v>0</v>
+        <v>16.22</v>
       </c>
       <c r="I44" s="2">
-        <v>8</v>
+        <v>7.3</v>
       </c>
       <c r="J44">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K44" s="1">
-        <v>32.43</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2377,22 +2377,22 @@
         <v>31</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="1">
         <v>96.88</v>
       </c>
       <c r="H46" s="1">
-        <v>0</v>
+        <v>3.13</v>
       </c>
       <c r="I46" s="2">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="J46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2482,22 +2482,22 @@
         <v>38</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
         <v>97.44</v>
       </c>
       <c r="H49" s="1">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="I49" s="2">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="J49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3144,13 +3144,13 @@
         <v>43</v>
       </c>
       <c r="E68">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F68">
         <v>10</v>
       </c>
       <c r="G68" s="1">
-        <v>74.42</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H68" s="1">
         <v>23.26</v>
@@ -3159,10 +3159,10 @@
         <v>7.2</v>
       </c>
       <c r="J68">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" s="1">
-        <v>2.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -3179,13 +3179,13 @@
         <v>34</v>
       </c>
       <c r="E69">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F69">
         <v>9</v>
       </c>
       <c r="G69" s="1">
-        <v>70.59</v>
+        <v>73.53</v>
       </c>
       <c r="H69" s="1">
         <v>26.47</v>
@@ -3194,10 +3194,10 @@
         <v>6.6</v>
       </c>
       <c r="J69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>2.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3214,25 +3214,25 @@
         <v>34</v>
       </c>
       <c r="E70">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F70">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G70" s="1">
-        <v>85.29000000000001</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="H70" s="1">
-        <v>2.94</v>
+        <v>11.76</v>
       </c>
       <c r="I70" s="2">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="J70">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K70" s="1">
-        <v>11.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -3249,25 +3249,25 @@
         <v>38</v>
       </c>
       <c r="E71">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F71">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G71" s="1">
-        <v>89.47</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="H71" s="1">
-        <v>0</v>
+        <v>5.26</v>
       </c>
       <c r="I71" s="2">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K71" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -3287,22 +3287,22 @@
         <v>29</v>
       </c>
       <c r="F72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G72" s="1">
         <v>90.63</v>
       </c>
       <c r="H72" s="1">
-        <v>3.13</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="I72" s="2">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="J72">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K72" s="1">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3319,25 +3319,25 @@
         <v>26</v>
       </c>
       <c r="E73">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G73" s="1">
-        <v>65.38</v>
+        <v>76.92</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>23.08</v>
       </c>
       <c r="I73" s="2">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="J73">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>34.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -3354,25 +3354,25 @@
         <v>33</v>
       </c>
       <c r="E74">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F74">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G74" s="1">
-        <v>81.81999999999999</v>
+        <v>84.84999999999999</v>
       </c>
       <c r="H74" s="1">
-        <v>0</v>
+        <v>15.15</v>
       </c>
       <c r="I74" s="2">
-        <v>9</v>
+        <v>8.4</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K74" s="1">
-        <v>18.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -3917,22 +3917,22 @@
         <v>23</v>
       </c>
       <c r="F90">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G90" s="1">
         <v>76.67</v>
       </c>
       <c r="H90" s="1">
-        <v>0</v>
+        <v>23.33</v>
       </c>
       <c r="I90" s="2">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="J90">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K90" s="1">
-        <v>23.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -3952,22 +3952,22 @@
         <v>31</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G91" s="1">
         <v>86.11</v>
       </c>
       <c r="H91" s="1">
-        <v>0</v>
+        <v>13.89</v>
       </c>
       <c r="I91" s="2">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="J91">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>13.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -4512,22 +4512,22 @@
         <v>33</v>
       </c>
       <c r="F107">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G107" s="1">
         <v>80.48999999999999</v>
       </c>
       <c r="H107" s="1">
-        <v>0</v>
+        <v>19.51</v>
       </c>
       <c r="I107" s="2">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="J107">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K107" s="1">
-        <v>19.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -4547,22 +4547,22 @@
         <v>32</v>
       </c>
       <c r="F108">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G108" s="1">
         <v>80</v>
       </c>
       <c r="H108" s="1">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="I108" s="2">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="J108">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -4582,22 +4582,22 @@
         <v>23</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G109" s="1">
         <v>63.89</v>
       </c>
       <c r="H109" s="1">
-        <v>0</v>
+        <v>36.11</v>
       </c>
       <c r="I109" s="2">
-        <v>6.9</v>
+        <v>6.2</v>
       </c>
       <c r="J109">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>36.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -4687,22 +4687,22 @@
         <v>36</v>
       </c>
       <c r="F112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G112" s="1">
         <v>92.31</v>
       </c>
       <c r="H112" s="1">
-        <v>0</v>
+        <v>7.69</v>
       </c>
       <c r="I112" s="2">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="J112">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K112" s="1">
-        <v>7.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:11">
@@ -5104,19 +5104,19 @@
         <v>35</v>
       </c>
       <c r="E124">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F124">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G124" s="1">
-        <v>80</v>
+        <v>82.86</v>
       </c>
       <c r="H124" s="1">
-        <v>20</v>
+        <v>17.14</v>
       </c>
       <c r="I124" s="2">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="J124">
         <v>0</v>
@@ -5839,25 +5839,25 @@
         <v>35</v>
       </c>
       <c r="E145">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F145">
         <v>0</v>
       </c>
       <c r="G145" s="1">
-        <v>94.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="H145" s="1">
         <v>0</v>
       </c>
       <c r="I145" s="2">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="J145">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K145" s="1">
-        <v>5.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -5944,25 +5944,25 @@
         <v>26</v>
       </c>
       <c r="E148">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F148">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G148" s="1">
-        <v>26.92</v>
+        <v>46.15</v>
       </c>
       <c r="H148" s="1">
-        <v>0</v>
+        <v>53.85</v>
       </c>
       <c r="I148" s="2">
-        <v>7.1</v>
+        <v>5.3</v>
       </c>
       <c r="J148">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>73.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -5979,25 +5979,25 @@
         <v>26</v>
       </c>
       <c r="E149">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G149" s="1">
-        <v>23.08</v>
+        <v>61.54</v>
       </c>
       <c r="H149" s="1">
-        <v>0</v>
+        <v>38.46</v>
       </c>
       <c r="I149" s="2">
-        <v>8.300000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="J149">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>76.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -6049,25 +6049,25 @@
         <v>36</v>
       </c>
       <c r="E151">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F151">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G151" s="1">
-        <v>30.56</v>
+        <v>80.56</v>
       </c>
       <c r="H151" s="1">
-        <v>0</v>
+        <v>19.44</v>
       </c>
       <c r="I151" s="2">
-        <v>7</v>
+        <v>7.4</v>
       </c>
       <c r="J151">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>69.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -6084,25 +6084,25 @@
         <v>40</v>
       </c>
       <c r="E152">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F152">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G152" s="1">
-        <v>25</v>
+        <v>77.5</v>
       </c>
       <c r="H152" s="1">
-        <v>0</v>
+        <v>22.5</v>
       </c>
       <c r="I152" s="2">
         <v>8.199999999999999</v>
       </c>
       <c r="J152">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -6119,25 +6119,25 @@
         <v>18</v>
       </c>
       <c r="E153">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F153">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G153" s="1">
-        <v>50</v>
+        <v>77.78</v>
       </c>
       <c r="H153" s="1">
-        <v>0</v>
+        <v>22.22</v>
       </c>
       <c r="I153" s="2">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="J153">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K153" s="1">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:11">
@@ -6367,22 +6367,22 @@
         <v>26</v>
       </c>
       <c r="F160">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G160" s="1">
         <v>96.3</v>
       </c>
       <c r="H160" s="1">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="I160" s="2">
-        <v>8.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="J160">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K160" s="1">
-        <v>3.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -6402,22 +6402,22 @@
         <v>11</v>
       </c>
       <c r="F161">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G161" s="1">
         <v>73.33</v>
       </c>
       <c r="H161" s="1">
-        <v>20</v>
+        <v>26.67</v>
       </c>
       <c r="I161" s="2">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="J161">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K161" s="1">
-        <v>6.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:11">
@@ -6437,22 +6437,22 @@
         <v>16</v>
       </c>
       <c r="F162">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G162" s="1">
         <v>76.19</v>
       </c>
       <c r="H162" s="1">
-        <v>9.52</v>
+        <v>23.81</v>
       </c>
       <c r="I162" s="2">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="J162">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K162" s="1">
-        <v>14.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:11">
@@ -7172,22 +7172,22 @@
         <v>33</v>
       </c>
       <c r="F183">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G183" s="1">
         <v>80.48999999999999</v>
       </c>
       <c r="H183" s="1">
-        <v>12.2</v>
+        <v>19.51</v>
       </c>
       <c r="I183" s="2">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="J183">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>7.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -7204,25 +7204,25 @@
         <v>40</v>
       </c>
       <c r="E184">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F184">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G184" s="1">
-        <v>77.5</v>
+        <v>80</v>
       </c>
       <c r="H184" s="1">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I184" s="2">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="J184">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K184" s="1">
-        <v>22.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:11">
@@ -7309,25 +7309,25 @@
         <v>34</v>
       </c>
       <c r="E187">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G187" s="1">
-        <v>76.47</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="H187" s="1">
-        <v>11.76</v>
+        <v>14.71</v>
       </c>
       <c r="I187" s="2">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="J187">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K187" s="1">
-        <v>11.76</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -7347,22 +7347,22 @@
         <v>31</v>
       </c>
       <c r="F188">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G188" s="1">
         <v>75.61</v>
       </c>
       <c r="H188" s="1">
-        <v>19.51</v>
+        <v>24.39</v>
       </c>
       <c r="I188" s="2">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="J188">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K188" s="1">
-        <v>4.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:11">
@@ -7379,25 +7379,25 @@
         <v>40</v>
       </c>
       <c r="E189">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F189">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G189" s="1">
-        <v>67.5</v>
+        <v>70</v>
       </c>
       <c r="H189" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I189" s="2">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="J189">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K189" s="1">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:11">
@@ -7417,22 +7417,22 @@
         <v>27</v>
       </c>
       <c r="F190">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G190" s="1">
         <v>75</v>
       </c>
       <c r="H190" s="1">
-        <v>22.22</v>
+        <v>25</v>
       </c>
       <c r="I190" s="2">
         <v>6.1</v>
       </c>
       <c r="J190">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K190" s="1">
-        <v>2.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" spans="1:11">
@@ -7452,22 +7452,22 @@
         <v>22</v>
       </c>
       <c r="F191">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G191" s="1">
         <v>84.62</v>
       </c>
       <c r="H191" s="1">
-        <v>0</v>
+        <v>15.38</v>
       </c>
       <c r="I191" s="2">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="J191">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K191" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" spans="1:11">
@@ -7554,25 +7554,25 @@
         <v>39</v>
       </c>
       <c r="E194">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F194">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G194" s="1">
-        <v>84.62</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="H194" s="1">
-        <v>0</v>
+        <v>10.26</v>
       </c>
       <c r="I194" s="2">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="J194">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K194" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195" spans="1:11">
@@ -7589,13 +7589,13 @@
         <v>39</v>
       </c>
       <c r="E195">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F195">
         <v>4</v>
       </c>
       <c r="G195" s="1">
-        <v>87.18000000000001</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="H195" s="1">
         <v>10.26</v>
@@ -7604,10 +7604,10 @@
         <v>7.2</v>
       </c>
       <c r="J195">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K195" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196" spans="1:11">
@@ -8481,25 +8481,25 @@
         <v>38</v>
       </c>
       <c r="E18">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G18" s="1">
-        <v>81.58</v>
+        <v>86.84</v>
       </c>
       <c r="H18" s="1">
-        <v>7.89</v>
+        <v>13.16</v>
       </c>
       <c r="I18" s="2">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -9149,22 +9149,22 @@
         <v>17</v>
       </c>
       <c r="F37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G37" s="1">
         <v>65.38</v>
       </c>
       <c r="H37" s="1">
-        <v>30.77</v>
+        <v>34.62</v>
       </c>
       <c r="I37" s="2">
         <v>7</v>
       </c>
       <c r="J37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="1">
-        <v>3.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -9181,25 +9181,25 @@
         <v>19</v>
       </c>
       <c r="E38">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G38" s="1">
-        <v>57.89</v>
+        <v>63.16</v>
       </c>
       <c r="H38" s="1">
-        <v>15.79</v>
+        <v>36.84</v>
       </c>
       <c r="I38" s="2">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="J38">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K38" s="1">
-        <v>26.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -9216,25 +9216,25 @@
         <v>34</v>
       </c>
       <c r="E39">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F39">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G39" s="1">
-        <v>64.70999999999999</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H39" s="1">
-        <v>17.65</v>
+        <v>32.35</v>
       </c>
       <c r="I39" s="2">
-        <v>7.4</v>
+        <v>6.9</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K39" s="1">
-        <v>17.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -9324,22 +9324,22 @@
         <v>33</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="1">
         <v>94.29000000000001</v>
       </c>
       <c r="H42" s="1">
-        <v>2.86</v>
+        <v>5.71</v>
       </c>
       <c r="I42" s="2">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="J42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" s="1">
-        <v>2.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -9356,25 +9356,25 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G43" s="1">
-        <v>52.38</v>
+        <v>90.48</v>
       </c>
       <c r="H43" s="1">
-        <v>0</v>
+        <v>9.52</v>
       </c>
       <c r="I43" s="2">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J43">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K43" s="1">
-        <v>47.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -9391,25 +9391,25 @@
         <v>37</v>
       </c>
       <c r="E44">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F44">
+        <v>6</v>
+      </c>
+      <c r="G44" s="1">
+        <v>81.08</v>
+      </c>
+      <c r="H44" s="1">
+        <v>16.22</v>
+      </c>
+      <c r="I44" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="J44">
         <v>1</v>
       </c>
-      <c r="G44" s="1">
-        <v>64.86</v>
-      </c>
-      <c r="H44" s="1">
+      <c r="K44" s="1">
         <v>2.7</v>
-      </c>
-      <c r="I44" s="2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="J44">
-        <v>12</v>
-      </c>
-      <c r="K44" s="1">
-        <v>32.43</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -9461,25 +9461,25 @@
         <v>32</v>
       </c>
       <c r="E46">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" s="1">
-        <v>90.63</v>
+        <v>96.88</v>
       </c>
       <c r="H46" s="1">
-        <v>6.25</v>
+        <v>3.13</v>
       </c>
       <c r="I46" s="2">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="J46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -9569,22 +9569,22 @@
         <v>38</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
         <v>97.44</v>
       </c>
       <c r="H49" s="1">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="I49" s="2">
         <v>6.5</v>
       </c>
       <c r="J49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -10231,13 +10231,13 @@
         <v>43</v>
       </c>
       <c r="E68">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F68">
         <v>10</v>
       </c>
       <c r="G68" s="1">
-        <v>74.42</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H68" s="1">
         <v>23.26</v>
@@ -10246,10 +10246,10 @@
         <v>6.4</v>
       </c>
       <c r="J68">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" s="1">
-        <v>2.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -10266,13 +10266,13 @@
         <v>34</v>
       </c>
       <c r="E69">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F69">
         <v>11</v>
       </c>
       <c r="G69" s="1">
-        <v>64.70999999999999</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H69" s="1">
         <v>32.35</v>
@@ -10281,10 +10281,10 @@
         <v>6.7</v>
       </c>
       <c r="J69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>2.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -10301,25 +10301,25 @@
         <v>34</v>
       </c>
       <c r="E70">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F70">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G70" s="1">
-        <v>50</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="H70" s="1">
-        <v>38.24</v>
+        <v>17.65</v>
       </c>
       <c r="I70" s="2">
-        <v>8.5</v>
+        <v>7.1</v>
       </c>
       <c r="J70">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K70" s="1">
-        <v>11.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -10336,25 +10336,25 @@
         <v>38</v>
       </c>
       <c r="E71">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F71">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G71" s="1">
-        <v>73.68000000000001</v>
+        <v>86.84</v>
       </c>
       <c r="H71" s="1">
-        <v>15.79</v>
+        <v>13.16</v>
       </c>
       <c r="I71" s="2">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K71" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -10371,25 +10371,25 @@
         <v>32</v>
       </c>
       <c r="E72">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G72" s="1">
-        <v>81.25</v>
+        <v>93.75</v>
       </c>
       <c r="H72" s="1">
-        <v>12.5</v>
+        <v>6.25</v>
       </c>
       <c r="I72" s="2">
-        <v>8.9</v>
+        <v>8.4</v>
       </c>
       <c r="J72">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K72" s="1">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -10406,25 +10406,25 @@
         <v>26</v>
       </c>
       <c r="E73">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F73">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G73" s="1">
-        <v>50</v>
+        <v>65.38</v>
       </c>
       <c r="H73" s="1">
-        <v>15.38</v>
+        <v>34.62</v>
       </c>
       <c r="I73" s="2">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="J73">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>34.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -10441,25 +10441,25 @@
         <v>33</v>
       </c>
       <c r="E74">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G74" s="1">
-        <v>72.73</v>
+        <v>87.88</v>
       </c>
       <c r="H74" s="1">
-        <v>9.09</v>
+        <v>12.12</v>
       </c>
       <c r="I74" s="2">
-        <v>9.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K74" s="1">
-        <v>18.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -11001,25 +11001,25 @@
         <v>30</v>
       </c>
       <c r="E90">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F90">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G90" s="1">
-        <v>63.33</v>
+        <v>66.67</v>
       </c>
       <c r="H90" s="1">
-        <v>13.33</v>
+        <v>33.33</v>
       </c>
       <c r="I90" s="2">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="J90">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K90" s="1">
-        <v>23.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -11036,25 +11036,25 @@
         <v>36</v>
       </c>
       <c r="E91">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F91">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G91" s="1">
-        <v>83.33</v>
+        <v>88.89</v>
       </c>
       <c r="H91" s="1">
-        <v>2.78</v>
+        <v>11.11</v>
       </c>
       <c r="I91" s="2">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="J91">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>13.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -11596,25 +11596,25 @@
         <v>41</v>
       </c>
       <c r="E107">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F107">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G107" s="1">
-        <v>75.61</v>
+        <v>78.05</v>
       </c>
       <c r="H107" s="1">
-        <v>4.88</v>
+        <v>21.95</v>
       </c>
       <c r="I107" s="2">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="J107">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K107" s="1">
-        <v>19.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -11634,22 +11634,22 @@
         <v>33</v>
       </c>
       <c r="F108">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G108" s="1">
         <v>82.5</v>
       </c>
       <c r="H108" s="1">
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="I108" s="2">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="J108">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -11666,25 +11666,25 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F109">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G109" s="1">
-        <v>52.78</v>
+        <v>61.11</v>
       </c>
       <c r="H109" s="1">
-        <v>11.11</v>
+        <v>38.89</v>
       </c>
       <c r="I109" s="2">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="J109">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>36.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -11771,25 +11771,25 @@
         <v>39</v>
       </c>
       <c r="E112">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112" s="1">
-        <v>92.31</v>
+        <v>97.44</v>
       </c>
       <c r="H112" s="1">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="I112" s="2">
         <v>7.8</v>
       </c>
       <c r="J112">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K112" s="1">
-        <v>7.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:11">
@@ -12926,13 +12926,13 @@
         <v>35</v>
       </c>
       <c r="E145">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F145">
         <v>0</v>
       </c>
       <c r="G145" s="1">
-        <v>94.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="H145" s="1">
         <v>0</v>
@@ -12941,10 +12941,10 @@
         <v>9</v>
       </c>
       <c r="J145">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K145" s="1">
-        <v>5.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -13031,25 +13031,25 @@
         <v>26</v>
       </c>
       <c r="E148">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F148">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G148" s="1">
-        <v>11.54</v>
+        <v>30.77</v>
       </c>
       <c r="H148" s="1">
-        <v>15.38</v>
+        <v>69.23</v>
       </c>
       <c r="I148" s="2">
-        <v>5.6</v>
+        <v>4.8</v>
       </c>
       <c r="J148">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>73.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -13066,25 +13066,25 @@
         <v>26</v>
       </c>
       <c r="E149">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G149" s="1">
-        <v>23.08</v>
+        <v>61.54</v>
       </c>
       <c r="H149" s="1">
-        <v>0</v>
+        <v>38.46</v>
       </c>
       <c r="I149" s="2">
-        <v>8.199999999999999</v>
+        <v>6.2</v>
       </c>
       <c r="J149">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>76.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -13136,25 +13136,25 @@
         <v>36</v>
       </c>
       <c r="E151">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F151">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G151" s="1">
-        <v>27.78</v>
+        <v>77.78</v>
       </c>
       <c r="H151" s="1">
-        <v>2.78</v>
+        <v>22.22</v>
       </c>
       <c r="I151" s="2">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
       <c r="J151">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>69.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -13171,25 +13171,25 @@
         <v>40</v>
       </c>
       <c r="E152">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F152">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G152" s="1">
-        <v>25</v>
+        <v>77.5</v>
       </c>
       <c r="H152" s="1">
-        <v>0</v>
+        <v>22.5</v>
       </c>
       <c r="I152" s="2">
-        <v>9.6</v>
+        <v>8.5</v>
       </c>
       <c r="J152">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -13206,25 +13206,25 @@
         <v>18</v>
       </c>
       <c r="E153">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F153">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G153" s="1">
-        <v>44.44</v>
+        <v>72.22</v>
       </c>
       <c r="H153" s="1">
-        <v>5.56</v>
+        <v>27.78</v>
       </c>
       <c r="I153" s="2">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="J153">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K153" s="1">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:11">
@@ -13454,22 +13454,22 @@
         <v>26</v>
       </c>
       <c r="F160">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G160" s="1">
         <v>96.3</v>
       </c>
       <c r="H160" s="1">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="I160" s="2">
         <v>7.7</v>
       </c>
       <c r="J160">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K160" s="1">
-        <v>3.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -13486,25 +13486,25 @@
         <v>15</v>
       </c>
       <c r="E161">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F161">
         <v>4</v>
       </c>
       <c r="G161" s="1">
-        <v>66.67</v>
+        <v>73.33</v>
       </c>
       <c r="H161" s="1">
         <v>26.67</v>
       </c>
       <c r="I161" s="2">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="J161">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K161" s="1">
-        <v>6.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:11">
@@ -13521,25 +13521,25 @@
         <v>21</v>
       </c>
       <c r="E162">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F162">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G162" s="1">
-        <v>85.70999999999999</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H162" s="1">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="I162" s="2">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="J162">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K162" s="1">
-        <v>14.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:11">
@@ -13941,16 +13941,16 @@
         <v>40</v>
       </c>
       <c r="E174">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F174">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G174" s="1">
-        <v>80</v>
+        <v>82.5</v>
       </c>
       <c r="H174" s="1">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="I174" s="2">
         <v>7.4</v>
@@ -14256,25 +14256,25 @@
         <v>41</v>
       </c>
       <c r="E183">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F183">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G183" s="1">
-        <v>78.05</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="H183" s="1">
-        <v>14.63</v>
+        <v>17.07</v>
       </c>
       <c r="I183" s="2">
         <v>6.4</v>
       </c>
       <c r="J183">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>7.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -14291,25 +14291,25 @@
         <v>40</v>
       </c>
       <c r="E184">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F184">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G184" s="1">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H184" s="1">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="I184" s="2">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="J184">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K184" s="1">
-        <v>22.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:11">
@@ -14396,25 +14396,25 @@
         <v>34</v>
       </c>
       <c r="E187">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F187">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G187" s="1">
-        <v>70.59</v>
+        <v>76.47</v>
       </c>
       <c r="H187" s="1">
-        <v>17.65</v>
+        <v>20.59</v>
       </c>
       <c r="I187" s="2">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="J187">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K187" s="1">
-        <v>11.76</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -14434,22 +14434,22 @@
         <v>27</v>
       </c>
       <c r="F188">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G188" s="1">
         <v>65.84999999999999</v>
       </c>
       <c r="H188" s="1">
-        <v>29.27</v>
+        <v>34.15</v>
       </c>
       <c r="I188" s="2">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="J188">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K188" s="1">
-        <v>4.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:11">
@@ -14466,25 +14466,25 @@
         <v>40</v>
       </c>
       <c r="E189">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F189">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G189" s="1">
-        <v>60</v>
+        <v>62.5</v>
       </c>
       <c r="H189" s="1">
-        <v>27.5</v>
+        <v>37.5</v>
       </c>
       <c r="I189" s="2">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="J189">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K189" s="1">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:11">
@@ -14504,22 +14504,22 @@
         <v>22</v>
       </c>
       <c r="F190">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G190" s="1">
         <v>61.11</v>
       </c>
       <c r="H190" s="1">
-        <v>36.11</v>
+        <v>38.89</v>
       </c>
       <c r="I190" s="2">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="J190">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K190" s="1">
-        <v>2.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" spans="1:11">
@@ -14539,22 +14539,22 @@
         <v>16</v>
       </c>
       <c r="F191">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G191" s="1">
         <v>61.54</v>
       </c>
       <c r="H191" s="1">
-        <v>23.08</v>
+        <v>38.46</v>
       </c>
       <c r="I191" s="2">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="J191">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K191" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" spans="1:11">
@@ -14641,25 +14641,25 @@
         <v>39</v>
       </c>
       <c r="E194">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F194">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G194" s="1">
-        <v>84.62</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="H194" s="1">
-        <v>0</v>
+        <v>10.26</v>
       </c>
       <c r="I194" s="2">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="J194">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K194" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195" spans="1:11">
@@ -14676,25 +14676,25 @@
         <v>39</v>
       </c>
       <c r="E195">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F195">
         <v>3</v>
       </c>
       <c r="G195" s="1">
-        <v>89.73999999999999</v>
+        <v>92.31</v>
       </c>
       <c r="H195" s="1">
         <v>7.69</v>
       </c>
       <c r="I195" s="2">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="J195">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K195" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196" spans="1:11">
@@ -15568,25 +15568,25 @@
         <v>38</v>
       </c>
       <c r="E18">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G18" s="1">
-        <v>81.58</v>
+        <v>86.84</v>
       </c>
       <c r="H18" s="1">
-        <v>7.89</v>
+        <v>13.16</v>
       </c>
       <c r="I18" s="2">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -16236,22 +16236,22 @@
         <v>17</v>
       </c>
       <c r="F37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G37" s="1">
         <v>65.38</v>
       </c>
       <c r="H37" s="1">
-        <v>30.77</v>
+        <v>34.62</v>
       </c>
       <c r="I37" s="2">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="J37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="1">
-        <v>3.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -16268,25 +16268,25 @@
         <v>19</v>
       </c>
       <c r="E38">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G38" s="1">
-        <v>57.89</v>
+        <v>63.16</v>
       </c>
       <c r="H38" s="1">
-        <v>15.79</v>
+        <v>36.84</v>
       </c>
       <c r="I38" s="2">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="J38">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K38" s="1">
-        <v>26.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -16306,22 +16306,22 @@
         <v>23</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G39" s="1">
         <v>67.65000000000001</v>
       </c>
       <c r="H39" s="1">
-        <v>14.71</v>
+        <v>32.35</v>
       </c>
       <c r="I39" s="2">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K39" s="1">
-        <v>17.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -16411,22 +16411,22 @@
         <v>33</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="1">
         <v>94.29000000000001</v>
       </c>
       <c r="H42" s="1">
-        <v>2.86</v>
+        <v>5.71</v>
       </c>
       <c r="I42" s="2">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="J42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" s="1">
-        <v>2.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -16443,25 +16443,25 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="1">
-        <v>52.38</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H43" s="1">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="I43" s="2">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J43">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K43" s="1">
-        <v>47.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -16478,25 +16478,25 @@
         <v>37</v>
       </c>
       <c r="E44">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G44" s="1">
-        <v>67.56999999999999</v>
+        <v>81.08</v>
       </c>
       <c r="H44" s="1">
-        <v>0</v>
+        <v>16.22</v>
       </c>
       <c r="I44" s="2">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
       <c r="J44">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K44" s="1">
-        <v>32.43</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -16548,25 +16548,25 @@
         <v>32</v>
       </c>
       <c r="E46">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F46">
         <v>1</v>
       </c>
       <c r="G46" s="1">
-        <v>93.75</v>
+        <v>96.88</v>
       </c>
       <c r="H46" s="1">
         <v>3.13</v>
       </c>
       <c r="I46" s="2">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="J46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -16656,22 +16656,22 @@
         <v>38</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
         <v>97.44</v>
       </c>
       <c r="H49" s="1">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="I49" s="2">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="J49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -17318,13 +17318,13 @@
         <v>43</v>
       </c>
       <c r="E68">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F68">
         <v>10</v>
       </c>
       <c r="G68" s="1">
-        <v>74.42</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H68" s="1">
         <v>23.26</v>
@@ -17333,10 +17333,10 @@
         <v>7</v>
       </c>
       <c r="J68">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" s="1">
-        <v>2.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -17353,13 +17353,13 @@
         <v>34</v>
       </c>
       <c r="E69">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F69">
         <v>11</v>
       </c>
       <c r="G69" s="1">
-        <v>64.70999999999999</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="H69" s="1">
         <v>32.35</v>
@@ -17368,10 +17368,10 @@
         <v>6.7</v>
       </c>
       <c r="J69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>2.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -17388,25 +17388,25 @@
         <v>34</v>
       </c>
       <c r="E70">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F70">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G70" s="1">
-        <v>85.29000000000001</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="H70" s="1">
-        <v>2.94</v>
+        <v>17.65</v>
       </c>
       <c r="I70" s="2">
-        <v>7.9</v>
+        <v>7.4</v>
       </c>
       <c r="J70">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K70" s="1">
-        <v>11.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -17423,25 +17423,25 @@
         <v>38</v>
       </c>
       <c r="E71">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F71">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G71" s="1">
-        <v>89.47</v>
+        <v>86.84</v>
       </c>
       <c r="H71" s="1">
-        <v>0</v>
+        <v>13.16</v>
       </c>
       <c r="I71" s="2">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K71" s="1">
-        <v>10.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -17461,22 +17461,22 @@
         <v>30</v>
       </c>
       <c r="F72">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G72" s="1">
         <v>93.75</v>
       </c>
       <c r="H72" s="1">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="I72" s="2">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="J72">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K72" s="1">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -17496,22 +17496,22 @@
         <v>17</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G73" s="1">
         <v>65.38</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>34.62</v>
       </c>
       <c r="I73" s="2">
-        <v>7.9</v>
+        <v>6.8</v>
       </c>
       <c r="J73">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>34.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -17528,25 +17528,25 @@
         <v>33</v>
       </c>
       <c r="E74">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F74">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G74" s="1">
-        <v>81.81999999999999</v>
+        <v>87.88</v>
       </c>
       <c r="H74" s="1">
-        <v>0</v>
+        <v>12.12</v>
       </c>
       <c r="I74" s="2">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K74" s="1">
-        <v>18.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -18088,25 +18088,25 @@
         <v>30</v>
       </c>
       <c r="E90">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F90">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G90" s="1">
-        <v>63.33</v>
+        <v>66.67</v>
       </c>
       <c r="H90" s="1">
-        <v>13.33</v>
+        <v>33.33</v>
       </c>
       <c r="I90" s="2">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
       <c r="J90">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K90" s="1">
-        <v>23.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -18123,25 +18123,25 @@
         <v>36</v>
       </c>
       <c r="E91">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F91">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G91" s="1">
-        <v>83.33</v>
+        <v>88.89</v>
       </c>
       <c r="H91" s="1">
-        <v>2.78</v>
+        <v>11.11</v>
       </c>
       <c r="I91" s="2">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="J91">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>13.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -18683,25 +18683,25 @@
         <v>41</v>
       </c>
       <c r="E107">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F107">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G107" s="1">
-        <v>75.61</v>
+        <v>78.05</v>
       </c>
       <c r="H107" s="1">
-        <v>4.88</v>
+        <v>21.95</v>
       </c>
       <c r="I107" s="2">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="J107">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K107" s="1">
-        <v>19.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -18721,22 +18721,22 @@
         <v>33</v>
       </c>
       <c r="F108">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G108" s="1">
         <v>82.5</v>
       </c>
       <c r="H108" s="1">
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="I108" s="2">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="J108">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -18753,25 +18753,25 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F109">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G109" s="1">
-        <v>52.78</v>
+        <v>61.11</v>
       </c>
       <c r="H109" s="1">
-        <v>11.11</v>
+        <v>38.89</v>
       </c>
       <c r="I109" s="2">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="J109">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>36.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -18858,25 +18858,25 @@
         <v>39</v>
       </c>
       <c r="E112">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112" s="1">
-        <v>92.31</v>
+        <v>97.44</v>
       </c>
       <c r="H112" s="1">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="I112" s="2">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="J112">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K112" s="1">
-        <v>7.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:11">
@@ -20013,13 +20013,13 @@
         <v>35</v>
       </c>
       <c r="E145">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F145">
         <v>0</v>
       </c>
       <c r="G145" s="1">
-        <v>94.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="H145" s="1">
         <v>0</v>
@@ -20028,10 +20028,10 @@
         <v>8.699999999999999</v>
       </c>
       <c r="J145">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K145" s="1">
-        <v>5.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -20118,25 +20118,25 @@
         <v>26</v>
       </c>
       <c r="E148">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F148">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G148" s="1">
-        <v>11.54</v>
+        <v>30.77</v>
       </c>
       <c r="H148" s="1">
-        <v>15.38</v>
+        <v>69.23</v>
       </c>
       <c r="I148" s="2">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="J148">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>73.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -20153,25 +20153,25 @@
         <v>26</v>
       </c>
       <c r="E149">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G149" s="1">
-        <v>23.08</v>
+        <v>61.54</v>
       </c>
       <c r="H149" s="1">
-        <v>0</v>
+        <v>38.46</v>
       </c>
       <c r="I149" s="2">
-        <v>8.5</v>
+        <v>6.6</v>
       </c>
       <c r="J149">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>76.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -20223,25 +20223,25 @@
         <v>36</v>
       </c>
       <c r="E151">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F151">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G151" s="1">
-        <v>27.78</v>
+        <v>77.78</v>
       </c>
       <c r="H151" s="1">
-        <v>2.78</v>
+        <v>22.22</v>
       </c>
       <c r="I151" s="2">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="J151">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>69.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -20258,25 +20258,25 @@
         <v>40</v>
       </c>
       <c r="E152">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F152">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G152" s="1">
-        <v>25</v>
+        <v>77.5</v>
       </c>
       <c r="H152" s="1">
-        <v>0</v>
+        <v>22.5</v>
       </c>
       <c r="I152" s="2">
-        <v>9.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="J152">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -20293,25 +20293,25 @@
         <v>18</v>
       </c>
       <c r="E153">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F153">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G153" s="1">
-        <v>44.44</v>
+        <v>72.22</v>
       </c>
       <c r="H153" s="1">
-        <v>5.56</v>
+        <v>27.78</v>
       </c>
       <c r="I153" s="2">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="J153">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K153" s="1">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:11">
@@ -20541,22 +20541,22 @@
         <v>26</v>
       </c>
       <c r="F160">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G160" s="1">
         <v>96.3</v>
       </c>
       <c r="H160" s="1">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="I160" s="2">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="J160">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K160" s="1">
-        <v>3.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -20573,25 +20573,25 @@
         <v>15</v>
       </c>
       <c r="E161">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F161">
         <v>4</v>
       </c>
       <c r="G161" s="1">
-        <v>66.67</v>
+        <v>73.33</v>
       </c>
       <c r="H161" s="1">
         <v>26.67</v>
       </c>
       <c r="I161" s="2">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="J161">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K161" s="1">
-        <v>6.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:11">
@@ -20608,25 +20608,25 @@
         <v>21</v>
       </c>
       <c r="E162">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F162">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G162" s="1">
-        <v>85.70999999999999</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="H162" s="1">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="I162" s="2">
-        <v>8.1</v>
+        <v>7.8</v>
       </c>
       <c r="J162">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K162" s="1">
-        <v>14.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:11">
@@ -21343,25 +21343,25 @@
         <v>41</v>
       </c>
       <c r="E183">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F183">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G183" s="1">
-        <v>78.05</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="H183" s="1">
-        <v>14.63</v>
+        <v>17.07</v>
       </c>
       <c r="I183" s="2">
         <v>6.6</v>
       </c>
       <c r="J183">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>7.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -21378,25 +21378,25 @@
         <v>40</v>
       </c>
       <c r="E184">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F184">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G184" s="1">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H184" s="1">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="I184" s="2">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="J184">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K184" s="1">
-        <v>22.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:11">
@@ -21483,25 +21483,25 @@
         <v>34</v>
       </c>
       <c r="E187">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F187">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G187" s="1">
-        <v>70.59</v>
+        <v>76.47</v>
       </c>
       <c r="H187" s="1">
-        <v>17.65</v>
+        <v>20.59</v>
       </c>
       <c r="I187" s="2">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="J187">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K187" s="1">
-        <v>11.76</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -21521,22 +21521,22 @@
         <v>27</v>
       </c>
       <c r="F188">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G188" s="1">
         <v>65.84999999999999</v>
       </c>
       <c r="H188" s="1">
-        <v>29.27</v>
+        <v>34.15</v>
       </c>
       <c r="I188" s="2">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="J188">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K188" s="1">
-        <v>4.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:11">
@@ -21553,25 +21553,25 @@
         <v>40</v>
       </c>
       <c r="E189">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F189">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G189" s="1">
-        <v>60</v>
+        <v>62.5</v>
       </c>
       <c r="H189" s="1">
-        <v>27.5</v>
+        <v>37.5</v>
       </c>
       <c r="I189" s="2">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="J189">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K189" s="1">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:11">
@@ -21591,22 +21591,22 @@
         <v>22</v>
       </c>
       <c r="F190">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G190" s="1">
         <v>61.11</v>
       </c>
       <c r="H190" s="1">
-        <v>36.11</v>
+        <v>38.89</v>
       </c>
       <c r="I190" s="2">
         <v>6.3</v>
       </c>
       <c r="J190">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K190" s="1">
-        <v>2.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" spans="1:11">
@@ -21626,22 +21626,22 @@
         <v>16</v>
       </c>
       <c r="F191">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G191" s="1">
         <v>61.54</v>
       </c>
       <c r="H191" s="1">
-        <v>23.08</v>
+        <v>38.46</v>
       </c>
       <c r="I191" s="2">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="J191">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K191" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" spans="1:11">
@@ -21728,25 +21728,25 @@
         <v>39</v>
       </c>
       <c r="E194">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F194">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G194" s="1">
-        <v>84.62</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="H194" s="1">
-        <v>0</v>
+        <v>10.26</v>
       </c>
       <c r="I194" s="2">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="J194">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K194" s="1">
-        <v>15.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195" spans="1:11">
@@ -21763,25 +21763,25 @@
         <v>39</v>
       </c>
       <c r="E195">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F195">
         <v>3</v>
       </c>
       <c r="G195" s="1">
-        <v>89.73999999999999</v>
+        <v>92.31</v>
       </c>
       <c r="H195" s="1">
         <v>7.69</v>
       </c>
       <c r="I195" s="2">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="J195">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K195" s="1">
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196" spans="1:11">

</xml_diff>

<commit_message>
Primer Parcial Media Noche
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -1440,22 +1440,25 @@
         <v>34</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G20" s="1">
-        <v>0</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="H20" s="1">
-        <v>0</v>
+        <v>11.76</v>
+      </c>
+      <c r="I20" s="2">
+        <v>7.3</v>
       </c>
       <c r="J20">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1822,22 +1825,25 @@
         <v>39</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" s="1">
-        <v>0</v>
+        <v>92.31</v>
       </c>
       <c r="H31" s="1">
-        <v>0</v>
+        <v>7.69</v>
+      </c>
+      <c r="I31" s="2">
+        <v>7.7</v>
       </c>
       <c r="J31">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K31" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2306,22 +2312,25 @@
         <v>41</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G45" s="1">
-        <v>0</v>
+        <v>92.68000000000001</v>
       </c>
       <c r="H45" s="1">
-        <v>0</v>
+        <v>7.32</v>
+      </c>
+      <c r="I45" s="2">
+        <v>8</v>
       </c>
       <c r="J45">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K45" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2863,22 +2872,25 @@
         <v>41</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G61" s="1">
-        <v>0</v>
+        <v>90.23999999999999</v>
       </c>
       <c r="H61" s="1">
-        <v>0</v>
+        <v>9.76</v>
+      </c>
+      <c r="I61" s="2">
+        <v>6.7</v>
       </c>
       <c r="J61">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K61" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3277,22 +3289,25 @@
         <v>38</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G73" s="1">
-        <v>0</v>
+        <v>81.58</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>18.42</v>
+      </c>
+      <c r="I73" s="2">
+        <v>6.3</v>
       </c>
       <c r="J73">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -3901,22 +3916,25 @@
         <v>32</v>
       </c>
       <c r="E91">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F91">
         <v>0</v>
       </c>
       <c r="G91" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H91" s="1">
         <v>0</v>
       </c>
+      <c r="I91" s="2">
+        <v>6.3</v>
+      </c>
       <c r="J91">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -4003,22 +4021,25 @@
         <v>29</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" s="1">
-        <v>0</v>
+        <v>96.55</v>
       </c>
       <c r="H94" s="1">
-        <v>0</v>
+        <v>3.45</v>
+      </c>
+      <c r="I94" s="2">
+        <v>6.1</v>
       </c>
       <c r="J94">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K94" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -4522,22 +4543,25 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G109" s="1">
-        <v>0</v>
+        <v>83.33</v>
       </c>
       <c r="H109" s="1">
-        <v>0</v>
+        <v>16.67</v>
+      </c>
+      <c r="I109" s="2">
+        <v>8</v>
       </c>
       <c r="J109">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -4799,25 +4823,25 @@
         <v>32</v>
       </c>
       <c r="E117">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F117">
         <v>0</v>
       </c>
       <c r="G117" s="1">
-        <v>96.88</v>
+        <v>100</v>
       </c>
       <c r="H117" s="1">
         <v>0</v>
       </c>
       <c r="I117" s="2">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="J117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K117" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:11">
@@ -4974,25 +4998,25 @@
         <v>31</v>
       </c>
       <c r="E122">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F122">
         <v>0</v>
       </c>
       <c r="G122" s="1">
-        <v>93.55</v>
+        <v>100</v>
       </c>
       <c r="H122" s="1">
         <v>0</v>
       </c>
       <c r="I122" s="2">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="J122">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K122" s="1">
-        <v>6.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:11">
@@ -5254,22 +5278,25 @@
         <v>43</v>
       </c>
       <c r="E130">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F130">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G130" s="1">
-        <v>0</v>
+        <v>74.42</v>
       </c>
       <c r="H130" s="1">
-        <v>0</v>
+        <v>25.58</v>
+      </c>
+      <c r="I130" s="2">
+        <v>6.7</v>
       </c>
       <c r="J130">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K130" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:11">
@@ -5286,22 +5313,25 @@
         <v>26</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>0</v>
+        <v>76.92</v>
       </c>
       <c r="H131" s="1">
-        <v>0</v>
+        <v>23.08</v>
+      </c>
+      <c r="I131" s="2">
+        <v>7.5</v>
       </c>
       <c r="J131">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K131" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:11">
@@ -5528,25 +5558,25 @@
         <v>30</v>
       </c>
       <c r="E138">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G138" s="1">
-        <v>63.33</v>
+        <v>93.33</v>
       </c>
       <c r="H138" s="1">
-        <v>0</v>
+        <v>3.33</v>
       </c>
       <c r="I138" s="2">
-        <v>8.6</v>
+        <v>7.9</v>
       </c>
       <c r="J138">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K138" s="1">
-        <v>33.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:11">
@@ -5563,25 +5593,25 @@
         <v>31</v>
       </c>
       <c r="E139">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F139">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G139" s="1">
-        <v>58.06</v>
+        <v>61.29</v>
       </c>
       <c r="H139" s="1">
-        <v>22.58</v>
+        <v>25.81</v>
       </c>
       <c r="I139" s="2">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="J139">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K139" s="1">
-        <v>12.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:11">
@@ -5613,10 +5643,10 @@
         <v>7.3</v>
       </c>
       <c r="J140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K140" s="1">
-        <v>3.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:11">
@@ -5668,22 +5698,25 @@
         <v>28</v>
       </c>
       <c r="E142">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F142">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G142" s="1">
-        <v>0</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="H142" s="1">
-        <v>0</v>
+        <v>10.71</v>
+      </c>
+      <c r="I142" s="2">
+        <v>7.7</v>
       </c>
       <c r="J142">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K142" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:11">
@@ -5700,25 +5733,25 @@
         <v>14</v>
       </c>
       <c r="E143">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F143">
         <v>0</v>
       </c>
       <c r="G143" s="1">
-        <v>64.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="H143" s="1">
         <v>0</v>
       </c>
       <c r="I143" s="2">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="J143">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>35.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -6155,25 +6188,25 @@
         <v>31</v>
       </c>
       <c r="E156">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F156">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G156" s="1">
-        <v>70.97</v>
+        <v>77.42</v>
       </c>
       <c r="H156" s="1">
-        <v>12.9</v>
+        <v>22.58</v>
       </c>
       <c r="I156" s="2">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="J156">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K156" s="1">
-        <v>16.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:11">
@@ -7030,22 +7063,25 @@
         <v>33</v>
       </c>
       <c r="E181">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F181">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G181" s="1">
-        <v>0</v>
+        <v>60.61</v>
       </c>
       <c r="H181" s="1">
-        <v>0</v>
+        <v>39.39</v>
+      </c>
+      <c r="I181" s="2">
+        <v>5.9</v>
       </c>
       <c r="J181">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K181" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -7237,22 +7273,25 @@
         <v>43</v>
       </c>
       <c r="E187">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F187">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G187" s="1">
-        <v>0</v>
+        <v>69.77</v>
       </c>
       <c r="H187" s="1">
-        <v>0</v>
+        <v>30.23</v>
+      </c>
+      <c r="I187" s="2">
+        <v>6.9</v>
       </c>
       <c r="J187">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K187" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -7584,22 +7623,25 @@
         <v>33</v>
       </c>
       <c r="E197">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F197">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G197" s="1">
-        <v>0</v>
+        <v>72.73</v>
       </c>
       <c r="H197" s="1">
-        <v>0</v>
+        <v>27.27</v>
+      </c>
+      <c r="I197" s="2">
+        <v>6.6</v>
       </c>
       <c r="J197">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -7616,22 +7658,25 @@
         <v>22</v>
       </c>
       <c r="E198">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F198">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G198" s="1">
-        <v>0</v>
+        <v>77.27</v>
       </c>
       <c r="H198" s="1">
-        <v>0</v>
+        <v>22.73</v>
+      </c>
+      <c r="I198" s="2">
+        <v>6.5</v>
       </c>
       <c r="J198">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -7648,22 +7693,25 @@
         <v>22</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F199">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G199" s="1">
-        <v>0</v>
+        <v>77.27</v>
       </c>
       <c r="H199" s="1">
-        <v>0</v>
+        <v>22.73</v>
+      </c>
+      <c r="I199" s="2">
+        <v>6.1</v>
       </c>
       <c r="J199">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">
@@ -8646,19 +8694,19 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="G20" s="1">
         <v>0</v>
       </c>
       <c r="H20" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J20">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -8998,19 +9046,19 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G31" s="1">
         <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J31">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K31" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -9446,19 +9494,19 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G45" s="1">
         <v>0</v>
       </c>
       <c r="H45" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J45">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K45" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -9958,19 +10006,19 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G61" s="1">
         <v>0</v>
       </c>
       <c r="H61" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J61">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K61" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -10342,19 +10390,19 @@
         <v>0</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G73" s="1">
         <v>0</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J73">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -10918,19 +10966,19 @@
         <v>0</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G91" s="1">
         <v>0</v>
       </c>
       <c r="H91" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J91">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -11014,19 +11062,19 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G94" s="1">
         <v>0</v>
       </c>
       <c r="H94" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J94">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K94" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -11494,19 +11542,19 @@
         <v>0</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G109" s="1">
         <v>0</v>
       </c>
       <c r="H109" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J109">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -11750,19 +11798,19 @@
         <v>0</v>
       </c>
       <c r="F117">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G117" s="1">
         <v>0</v>
       </c>
       <c r="H117" s="1">
-        <v>96.88</v>
+        <v>100</v>
       </c>
       <c r="J117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K117" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:11">
@@ -11910,19 +11958,19 @@
         <v>0</v>
       </c>
       <c r="F122">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G122" s="1">
         <v>0</v>
       </c>
       <c r="H122" s="1">
-        <v>93.55</v>
+        <v>100</v>
       </c>
       <c r="J122">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K122" s="1">
-        <v>6.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:11">
@@ -12166,19 +12214,19 @@
         <v>0</v>
       </c>
       <c r="F130">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G130" s="1">
         <v>0</v>
       </c>
       <c r="H130" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J130">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K130" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:11">
@@ -12198,19 +12246,19 @@
         <v>0</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G131" s="1">
         <v>0</v>
       </c>
       <c r="H131" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J131">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K131" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:11">
@@ -12422,19 +12470,19 @@
         <v>0</v>
       </c>
       <c r="F138">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G138" s="1">
         <v>0</v>
       </c>
       <c r="H138" s="1">
-        <v>63.33</v>
+        <v>96.67</v>
       </c>
       <c r="J138">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K138" s="1">
-        <v>33.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:11">
@@ -12454,19 +12502,19 @@
         <v>0</v>
       </c>
       <c r="F139">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G139" s="1">
         <v>0</v>
       </c>
       <c r="H139" s="1">
-        <v>80.65000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J139">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K139" s="1">
-        <v>12.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:11">
@@ -12495,10 +12543,10 @@
         <v>96.97</v>
       </c>
       <c r="J140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K140" s="1">
-        <v>3.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:11">
@@ -12550,19 +12598,19 @@
         <v>0</v>
       </c>
       <c r="F142">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G142" s="1">
         <v>0</v>
       </c>
       <c r="H142" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J142">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K142" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:11">
@@ -12582,19 +12630,19 @@
         <v>0</v>
       </c>
       <c r="F143">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G143" s="1">
         <v>0</v>
       </c>
       <c r="H143" s="1">
-        <v>64.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="J143">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>35.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -12998,19 +13046,19 @@
         <v>0</v>
       </c>
       <c r="F156">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G156" s="1">
         <v>0</v>
       </c>
       <c r="H156" s="1">
-        <v>83.87</v>
+        <v>100</v>
       </c>
       <c r="J156">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K156" s="1">
-        <v>16.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:11">
@@ -13798,19 +13846,19 @@
         <v>0</v>
       </c>
       <c r="F181">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="G181" s="1">
         <v>0</v>
       </c>
       <c r="H181" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J181">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K181" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -13990,19 +14038,19 @@
         <v>0</v>
       </c>
       <c r="F187">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G187" s="1">
         <v>0</v>
       </c>
       <c r="H187" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J187">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K187" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -14310,19 +14358,19 @@
         <v>0</v>
       </c>
       <c r="F197">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="G197" s="1">
         <v>0</v>
       </c>
       <c r="H197" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J197">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -14342,19 +14390,19 @@
         <v>0</v>
       </c>
       <c r="F198">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G198" s="1">
         <v>0</v>
       </c>
       <c r="H198" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J198">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -14374,19 +14422,19 @@
         <v>0</v>
       </c>
       <c r="F199">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G199" s="1">
         <v>0</v>
       </c>
       <c r="H199" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J199">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">
@@ -15405,22 +15453,25 @@
         <v>34</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G20" s="1">
-        <v>0</v>
+        <v>88.23999999999999</v>
       </c>
       <c r="H20" s="1">
-        <v>0</v>
+        <v>11.76</v>
+      </c>
+      <c r="I20" s="2">
+        <v>7.3</v>
       </c>
       <c r="J20">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -15787,22 +15838,25 @@
         <v>39</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" s="1">
-        <v>0</v>
+        <v>92.31</v>
       </c>
       <c r="H31" s="1">
-        <v>0</v>
+        <v>7.69</v>
+      </c>
+      <c r="I31" s="2">
+        <v>7.7</v>
       </c>
       <c r="J31">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K31" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -16271,22 +16325,25 @@
         <v>41</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G45" s="1">
-        <v>0</v>
+        <v>92.68000000000001</v>
       </c>
       <c r="H45" s="1">
-        <v>0</v>
+        <v>7.32</v>
+      </c>
+      <c r="I45" s="2">
+        <v>8</v>
       </c>
       <c r="J45">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K45" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -16828,22 +16885,25 @@
         <v>41</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G61" s="1">
-        <v>0</v>
+        <v>90.23999999999999</v>
       </c>
       <c r="H61" s="1">
-        <v>0</v>
+        <v>9.76</v>
+      </c>
+      <c r="I61" s="2">
+        <v>6.8</v>
       </c>
       <c r="J61">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K61" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -17242,22 +17302,25 @@
         <v>38</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G73" s="1">
-        <v>0</v>
+        <v>81.58</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>18.42</v>
+      </c>
+      <c r="I73" s="2">
+        <v>6.7</v>
       </c>
       <c r="J73">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K73" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -17866,22 +17929,25 @@
         <v>32</v>
       </c>
       <c r="E91">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F91">
         <v>0</v>
       </c>
       <c r="G91" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H91" s="1">
         <v>0</v>
       </c>
+      <c r="I91" s="2">
+        <v>6.3</v>
+      </c>
       <c r="J91">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -17968,22 +18034,25 @@
         <v>29</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" s="1">
-        <v>0</v>
+        <v>96.55</v>
       </c>
       <c r="H94" s="1">
-        <v>0</v>
+        <v>3.45</v>
+      </c>
+      <c r="I94" s="2">
+        <v>6.1</v>
       </c>
       <c r="J94">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K94" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -18487,22 +18556,25 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G109" s="1">
-        <v>0</v>
+        <v>83.33</v>
       </c>
       <c r="H109" s="1">
-        <v>0</v>
+        <v>16.67</v>
+      </c>
+      <c r="I109" s="2">
+        <v>8</v>
       </c>
       <c r="J109">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -18764,25 +18836,25 @@
         <v>32</v>
       </c>
       <c r="E117">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F117">
         <v>0</v>
       </c>
       <c r="G117" s="1">
-        <v>96.88</v>
+        <v>100</v>
       </c>
       <c r="H117" s="1">
         <v>0</v>
       </c>
       <c r="I117" s="2">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="J117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K117" s="1">
-        <v>3.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:11">
@@ -18939,25 +19011,25 @@
         <v>31</v>
       </c>
       <c r="E122">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F122">
         <v>0</v>
       </c>
       <c r="G122" s="1">
-        <v>93.55</v>
+        <v>100</v>
       </c>
       <c r="H122" s="1">
         <v>0</v>
       </c>
       <c r="I122" s="2">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="J122">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K122" s="1">
-        <v>6.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:11">
@@ -19219,22 +19291,25 @@
         <v>43</v>
       </c>
       <c r="E130">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F130">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G130" s="1">
-        <v>0</v>
+        <v>74.42</v>
       </c>
       <c r="H130" s="1">
-        <v>0</v>
+        <v>25.58</v>
+      </c>
+      <c r="I130" s="2">
+        <v>6.7</v>
       </c>
       <c r="J130">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K130" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:11">
@@ -19251,22 +19326,25 @@
         <v>26</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>0</v>
+        <v>76.92</v>
       </c>
       <c r="H131" s="1">
-        <v>0</v>
+        <v>23.08</v>
+      </c>
+      <c r="I131" s="2">
+        <v>7.5</v>
       </c>
       <c r="J131">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K131" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:11">
@@ -19493,25 +19571,25 @@
         <v>30</v>
       </c>
       <c r="E138">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F138">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G138" s="1">
-        <v>63.33</v>
+        <v>93.33</v>
       </c>
       <c r="H138" s="1">
-        <v>3.33</v>
+        <v>6.67</v>
       </c>
       <c r="I138" s="2">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
       <c r="J138">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K138" s="1">
-        <v>33.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:11">
@@ -19528,25 +19606,25 @@
         <v>31</v>
       </c>
       <c r="E139">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F139">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G139" s="1">
-        <v>58.06</v>
+        <v>61.29</v>
       </c>
       <c r="H139" s="1">
-        <v>29.03</v>
+        <v>38.71</v>
       </c>
       <c r="I139" s="2">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="J139">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K139" s="1">
-        <v>12.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:11">
@@ -19566,22 +19644,22 @@
         <v>30</v>
       </c>
       <c r="F140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G140" s="1">
         <v>90.91</v>
       </c>
       <c r="H140" s="1">
-        <v>6.06</v>
+        <v>9.09</v>
       </c>
       <c r="I140" s="2">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="J140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K140" s="1">
-        <v>3.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:11">
@@ -19633,22 +19711,25 @@
         <v>28</v>
       </c>
       <c r="E142">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F142">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G142" s="1">
-        <v>0</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="H142" s="1">
-        <v>0</v>
+        <v>10.71</v>
+      </c>
+      <c r="I142" s="2">
+        <v>7.7</v>
       </c>
       <c r="J142">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K142" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:11">
@@ -19665,25 +19746,25 @@
         <v>14</v>
       </c>
       <c r="E143">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F143">
         <v>0</v>
       </c>
       <c r="G143" s="1">
-        <v>64.29000000000001</v>
+        <v>100</v>
       </c>
       <c r="H143" s="1">
         <v>0</v>
       </c>
       <c r="I143" s="2">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="J143">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>35.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -20120,25 +20201,25 @@
         <v>31</v>
       </c>
       <c r="E156">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F156">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G156" s="1">
-        <v>70.97</v>
+        <v>77.42</v>
       </c>
       <c r="H156" s="1">
-        <v>12.9</v>
+        <v>22.58</v>
       </c>
       <c r="I156" s="2">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="J156">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K156" s="1">
-        <v>16.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:11">
@@ -20995,22 +21076,25 @@
         <v>33</v>
       </c>
       <c r="E181">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F181">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G181" s="1">
-        <v>0</v>
+        <v>60.61</v>
       </c>
       <c r="H181" s="1">
-        <v>0</v>
+        <v>39.39</v>
+      </c>
+      <c r="I181" s="2">
+        <v>5.9</v>
       </c>
       <c r="J181">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K181" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -21202,22 +21286,25 @@
         <v>43</v>
       </c>
       <c r="E187">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F187">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G187" s="1">
-        <v>0</v>
+        <v>69.77</v>
       </c>
       <c r="H187" s="1">
-        <v>0</v>
+        <v>30.23</v>
+      </c>
+      <c r="I187" s="2">
+        <v>6.9</v>
       </c>
       <c r="J187">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K187" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:11">
@@ -21549,22 +21636,25 @@
         <v>33</v>
       </c>
       <c r="E197">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F197">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G197" s="1">
-        <v>0</v>
+        <v>72.73</v>
       </c>
       <c r="H197" s="1">
-        <v>0</v>
+        <v>27.27</v>
+      </c>
+      <c r="I197" s="2">
+        <v>6.6</v>
       </c>
       <c r="J197">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -21581,22 +21671,25 @@
         <v>22</v>
       </c>
       <c r="E198">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F198">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G198" s="1">
-        <v>0</v>
+        <v>77.27</v>
       </c>
       <c r="H198" s="1">
-        <v>0</v>
+        <v>22.73</v>
+      </c>
+      <c r="I198" s="2">
+        <v>6.5</v>
       </c>
       <c r="J198">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -21613,22 +21706,25 @@
         <v>22</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F199">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G199" s="1">
-        <v>0</v>
+        <v>77.27</v>
       </c>
       <c r="H199" s="1">
-        <v>0</v>
+        <v>22.73</v>
+      </c>
+      <c r="I199" s="2">
+        <v>6.1</v>
       </c>
       <c r="J199">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">

</xml_diff>

<commit_message>
Primer Parcial 16 Mar Mañana
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -1965,22 +1965,25 @@
         <v>40</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="1">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H35" s="1">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="I35" s="2">
+        <v>8.199999999999999</v>
       </c>
       <c r="J35">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K35" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3152,22 +3155,25 @@
         <v>38</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G69" s="1">
-        <v>0</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="H69" s="1">
-        <v>0</v>
+        <v>5.26</v>
+      </c>
+      <c r="I69" s="2">
+        <v>9.199999999999999</v>
       </c>
       <c r="J69">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3429,22 +3435,25 @@
         <v>28</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G77" s="1">
-        <v>0</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="H77" s="1">
-        <v>0</v>
+        <v>21.43</v>
+      </c>
+      <c r="I77" s="2">
+        <v>6.1</v>
       </c>
       <c r="J77">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K77" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -4511,22 +4520,25 @@
         <v>36</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H108" s="1">
         <v>0</v>
       </c>
+      <c r="I108" s="2">
+        <v>9.1</v>
+      </c>
       <c r="J108">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -7798,22 +7810,25 @@
         <v>30</v>
       </c>
       <c r="E202">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F202">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G202" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H202" s="1">
-        <v>0</v>
+        <v>66.67</v>
+      </c>
+      <c r="I202" s="2">
+        <v>4.8</v>
       </c>
       <c r="J202">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K202" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:11">
@@ -7830,22 +7845,25 @@
         <v>30</v>
       </c>
       <c r="E203">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F203">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G203" s="1">
-        <v>0</v>
+        <v>36.67</v>
       </c>
       <c r="H203" s="1">
-        <v>0</v>
+        <v>63.33</v>
+      </c>
+      <c r="I203" s="2">
+        <v>5</v>
       </c>
       <c r="J203">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K203" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:11">
@@ -7862,22 +7880,25 @@
         <v>33</v>
       </c>
       <c r="E204">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F204">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G204" s="1">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="H204" s="1">
-        <v>0</v>
+        <v>33.33</v>
+      </c>
+      <c r="I204" s="2">
+        <v>6.8</v>
       </c>
       <c r="J204">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K204" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -7894,22 +7915,25 @@
         <v>33</v>
       </c>
       <c r="E205">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F205">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G205" s="1">
-        <v>0</v>
+        <v>54.55</v>
       </c>
       <c r="H205" s="1">
-        <v>0</v>
+        <v>45.45</v>
+      </c>
+      <c r="I205" s="2">
+        <v>5.8</v>
       </c>
       <c r="J205">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K205" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206" spans="1:11">
@@ -7926,22 +7950,25 @@
         <v>25</v>
       </c>
       <c r="E206">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F206">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G206" s="1">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H206" s="1">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="I206" s="2">
+        <v>5.7</v>
       </c>
       <c r="J206">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="K206" s="1">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207" spans="1:11">
@@ -9174,19 +9201,19 @@
         <v>0</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G35" s="1">
         <v>0</v>
       </c>
       <c r="H35" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J35">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K35" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -10262,19 +10289,19 @@
         <v>0</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G69" s="1">
         <v>0</v>
       </c>
       <c r="H69" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J69">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -10518,19 +10545,19 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G77" s="1">
         <v>0</v>
       </c>
       <c r="H77" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J77">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K77" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -11510,19 +11537,19 @@
         <v>0</v>
       </c>
       <c r="F108">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G108" s="1">
         <v>0</v>
       </c>
       <c r="H108" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J108">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -14518,19 +14545,19 @@
         <v>0</v>
       </c>
       <c r="F202">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G202" s="1">
         <v>0</v>
       </c>
       <c r="H202" s="1">
-        <v>0</v>
+        <v>96.67</v>
       </c>
       <c r="J202">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K202" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:11">
@@ -14550,19 +14577,19 @@
         <v>0</v>
       </c>
       <c r="F203">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G203" s="1">
         <v>0</v>
       </c>
       <c r="H203" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J203">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K203" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:11">
@@ -14582,19 +14609,19 @@
         <v>0</v>
       </c>
       <c r="F204">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="G204" s="1">
         <v>0</v>
       </c>
       <c r="H204" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J204">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K204" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -14614,19 +14641,19 @@
         <v>0</v>
       </c>
       <c r="F205">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="G205" s="1">
         <v>0</v>
       </c>
       <c r="H205" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J205">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K205" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206" spans="1:11">
@@ -14646,19 +14673,19 @@
         <v>0</v>
       </c>
       <c r="F206">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G206" s="1">
         <v>0</v>
       </c>
       <c r="H206" s="1">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="J206">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="K206" s="1">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207" spans="1:11">
@@ -15978,22 +16005,25 @@
         <v>40</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="1">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H35" s="1">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="I35" s="2">
+        <v>8.199999999999999</v>
       </c>
       <c r="J35">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K35" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -17165,22 +17195,25 @@
         <v>38</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G69" s="1">
-        <v>0</v>
+        <v>94.73999999999999</v>
       </c>
       <c r="H69" s="1">
-        <v>0</v>
+        <v>5.26</v>
+      </c>
+      <c r="I69" s="2">
+        <v>9.199999999999999</v>
       </c>
       <c r="J69">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -17442,22 +17475,25 @@
         <v>28</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G77" s="1">
-        <v>0</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="H77" s="1">
-        <v>0</v>
+        <v>21.43</v>
+      </c>
+      <c r="I77" s="2">
+        <v>6.2</v>
       </c>
       <c r="J77">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K77" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -18524,22 +18560,25 @@
         <v>36</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H108" s="1">
         <v>0</v>
       </c>
+      <c r="I108" s="2">
+        <v>9.1</v>
+      </c>
       <c r="J108">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -21811,22 +21850,25 @@
         <v>30</v>
       </c>
       <c r="E202">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F202">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G202" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H202" s="1">
-        <v>0</v>
+        <v>70</v>
+      </c>
+      <c r="I202" s="2">
+        <v>5.5</v>
       </c>
       <c r="J202">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K202" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:11">
@@ -21843,22 +21885,25 @@
         <v>30</v>
       </c>
       <c r="E203">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F203">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G203" s="1">
-        <v>0</v>
+        <v>36.67</v>
       </c>
       <c r="H203" s="1">
-        <v>0</v>
+        <v>63.33</v>
+      </c>
+      <c r="I203" s="2">
+        <v>5.6</v>
       </c>
       <c r="J203">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K203" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:11">
@@ -21875,22 +21920,25 @@
         <v>33</v>
       </c>
       <c r="E204">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F204">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G204" s="1">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="H204" s="1">
-        <v>0</v>
+        <v>33.33</v>
+      </c>
+      <c r="I204" s="2">
+        <v>6.9</v>
       </c>
       <c r="J204">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K204" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -21907,22 +21955,25 @@
         <v>33</v>
       </c>
       <c r="E205">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F205">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G205" s="1">
-        <v>0</v>
+        <v>54.55</v>
       </c>
       <c r="H205" s="1">
-        <v>0</v>
+        <v>45.45</v>
+      </c>
+      <c r="I205" s="2">
+        <v>6.1</v>
       </c>
       <c r="J205">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K205" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206" spans="1:11">
@@ -21939,22 +21990,25 @@
         <v>25</v>
       </c>
       <c r="E206">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F206">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G206" s="1">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H206" s="1">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="I206" s="2">
+        <v>6.1</v>
       </c>
       <c r="J206">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="K206" s="1">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207" spans="1:11">

</xml_diff>

<commit_message>
Primer Parcial con Totales Academia
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -1325,19 +1325,19 @@
         <v>101</v>
       </c>
       <c r="D15">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F15">
         <v>11</v>
       </c>
       <c r="G15" s="1">
-        <v>73.17</v>
+        <v>73.81</v>
       </c>
       <c r="H15" s="1">
-        <v>26.83</v>
+        <v>26.19</v>
       </c>
       <c r="I15" s="2">
         <v>6.4</v>
@@ -1745,22 +1745,22 @@
         <v>108</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E27">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F27">
         <v>19</v>
       </c>
       <c r="G27" s="1">
-        <v>54.76</v>
+        <v>53.66</v>
       </c>
       <c r="H27" s="1">
-        <v>45.24</v>
+        <v>46.34</v>
       </c>
       <c r="I27" s="2">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -2445,19 +2445,19 @@
         <v>101</v>
       </c>
       <c r="D47">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E47">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F47">
         <v>11</v>
       </c>
       <c r="G47" s="1">
-        <v>74.42</v>
+        <v>73.81</v>
       </c>
       <c r="H47" s="1">
-        <v>25.58</v>
+        <v>26.19</v>
       </c>
       <c r="I47" s="2">
         <v>6.7</v>
@@ -2900,22 +2900,22 @@
         <v>108</v>
       </c>
       <c r="D60">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E60">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
       <c r="G60" s="1">
-        <v>82.93000000000001</v>
+        <v>83.33</v>
       </c>
       <c r="H60" s="1">
-        <v>17.07</v>
+        <v>16.67</v>
       </c>
       <c r="I60" s="2">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="J60">
         <v>0</v>
@@ -3215,22 +3215,22 @@
         <v>121</v>
       </c>
       <c r="D69">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E69">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F69">
         <v>17</v>
       </c>
       <c r="G69" s="1">
-        <v>59.52</v>
+        <v>58.54</v>
       </c>
       <c r="H69" s="1">
-        <v>40.48</v>
+        <v>41.46</v>
       </c>
       <c r="I69" s="2">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="J69">
         <v>0</v>
@@ -3915,19 +3915,19 @@
         <v>125</v>
       </c>
       <c r="D89">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E89">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F89">
         <v>14</v>
       </c>
       <c r="G89" s="1">
-        <v>65.84999999999999</v>
+        <v>66.67</v>
       </c>
       <c r="H89" s="1">
-        <v>34.15</v>
+        <v>33.33</v>
       </c>
       <c r="I89" s="2">
         <v>6.6</v>
@@ -4335,19 +4335,19 @@
         <v>119</v>
       </c>
       <c r="D101">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E101">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F101">
         <v>7</v>
       </c>
       <c r="G101" s="1">
-        <v>82.93000000000001</v>
+        <v>83.33</v>
       </c>
       <c r="H101" s="1">
-        <v>17.07</v>
+        <v>16.67</v>
       </c>
       <c r="I101" s="2">
         <v>7.5</v>
@@ -4965,19 +4965,19 @@
         <v>125</v>
       </c>
       <c r="D119">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E119">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F119">
         <v>8</v>
       </c>
       <c r="G119" s="1">
-        <v>80.48999999999999</v>
+        <v>80</v>
       </c>
       <c r="H119" s="1">
-        <v>19.51</v>
+        <v>20</v>
       </c>
       <c r="I119" s="2">
         <v>7</v>
@@ -5805,22 +5805,22 @@
         <v>122</v>
       </c>
       <c r="D143">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E143">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F143">
         <v>3</v>
       </c>
       <c r="G143" s="1">
-        <v>92.86</v>
+        <v>92.68000000000001</v>
       </c>
       <c r="H143" s="1">
-        <v>7.14</v>
+        <v>7.32</v>
       </c>
       <c r="I143" s="2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J143">
         <v>0</v>
@@ -6365,19 +6365,19 @@
         <v>119</v>
       </c>
       <c r="D159">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E159">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F159">
         <v>13</v>
       </c>
       <c r="G159" s="1">
-        <v>69.77</v>
+        <v>69.05</v>
       </c>
       <c r="H159" s="1">
-        <v>30.23</v>
+        <v>30.95</v>
       </c>
       <c r="I159" s="2">
         <v>6.9</v>
@@ -6750,22 +6750,22 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E170">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F170">
         <v>9</v>
       </c>
       <c r="G170" s="1">
-        <v>78.05</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="H170" s="1">
-        <v>21.95</v>
+        <v>21.43</v>
       </c>
       <c r="I170" s="2">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="J170">
         <v>0</v>
@@ -6960,22 +6960,22 @@
         <v>122</v>
       </c>
       <c r="D176">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E176">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F176">
         <v>3</v>
       </c>
       <c r="G176" s="1">
-        <v>92.68000000000001</v>
+        <v>92.86</v>
       </c>
       <c r="H176" s="1">
-        <v>7.32</v>
+        <v>7.14</v>
       </c>
       <c r="I176" s="2">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="J176">
         <v>0</v>
@@ -8618,13 +8618,13 @@
         <v>101</v>
       </c>
       <c r="D15">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G15" s="1">
         <v>0</v>
@@ -9002,13 +9002,13 @@
         <v>108</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
       <c r="F27">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G27" s="1">
         <v>0</v>
@@ -9642,13 +9642,13 @@
         <v>101</v>
       </c>
       <c r="D47">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E47">
         <v>0</v>
       </c>
       <c r="F47">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G47" s="1">
         <v>0</v>
@@ -10058,13 +10058,13 @@
         <v>108</v>
       </c>
       <c r="D60">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E60">
         <v>0</v>
       </c>
       <c r="F60">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G60" s="1">
         <v>0</v>
@@ -10346,13 +10346,13 @@
         <v>121</v>
       </c>
       <c r="D69">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E69">
         <v>0</v>
       </c>
       <c r="F69">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G69" s="1">
         <v>0</v>
@@ -10986,13 +10986,13 @@
         <v>125</v>
       </c>
       <c r="D89">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E89">
         <v>0</v>
       </c>
       <c r="F89">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G89" s="1">
         <v>0</v>
@@ -11370,13 +11370,13 @@
         <v>119</v>
       </c>
       <c r="D101">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E101">
         <v>0</v>
       </c>
       <c r="F101">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G101" s="1">
         <v>0</v>
@@ -11946,13 +11946,13 @@
         <v>125</v>
       </c>
       <c r="D119">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E119">
         <v>0</v>
       </c>
       <c r="F119">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G119" s="1">
         <v>0</v>
@@ -12714,13 +12714,13 @@
         <v>122</v>
       </c>
       <c r="D143">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E143">
         <v>0</v>
       </c>
       <c r="F143">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G143" s="1">
         <v>0</v>
@@ -13226,13 +13226,13 @@
         <v>119</v>
       </c>
       <c r="D159">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E159">
         <v>0</v>
       </c>
       <c r="F159">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G159" s="1">
         <v>0</v>
@@ -13578,13 +13578,13 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E170">
         <v>0</v>
       </c>
       <c r="F170">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G170" s="1">
         <v>0</v>
@@ -13770,13 +13770,13 @@
         <v>122</v>
       </c>
       <c r="D176">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E176">
         <v>0</v>
       </c>
       <c r="F176">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G176" s="1">
         <v>0</v>
@@ -15365,19 +15365,19 @@
         <v>101</v>
       </c>
       <c r="D15">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F15">
         <v>11</v>
       </c>
       <c r="G15" s="1">
-        <v>73.17</v>
+        <v>73.81</v>
       </c>
       <c r="H15" s="1">
-        <v>26.83</v>
+        <v>26.19</v>
       </c>
       <c r="I15" s="2">
         <v>6.7</v>
@@ -15785,22 +15785,22 @@
         <v>108</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E27">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F27">
         <v>19</v>
       </c>
       <c r="G27" s="1">
-        <v>54.76</v>
+        <v>53.66</v>
       </c>
       <c r="H27" s="1">
-        <v>45.24</v>
+        <v>46.34</v>
       </c>
       <c r="I27" s="2">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -16485,19 +16485,19 @@
         <v>101</v>
       </c>
       <c r="D47">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E47">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F47">
         <v>11</v>
       </c>
       <c r="G47" s="1">
-        <v>74.42</v>
+        <v>73.81</v>
       </c>
       <c r="H47" s="1">
-        <v>25.58</v>
+        <v>26.19</v>
       </c>
       <c r="I47" s="2">
         <v>6.7</v>
@@ -16940,22 +16940,22 @@
         <v>108</v>
       </c>
       <c r="D60">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E60">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
       <c r="G60" s="1">
-        <v>82.93000000000001</v>
+        <v>83.33</v>
       </c>
       <c r="H60" s="1">
-        <v>17.07</v>
+        <v>16.67</v>
       </c>
       <c r="I60" s="2">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="J60">
         <v>0</v>
@@ -17255,22 +17255,22 @@
         <v>121</v>
       </c>
       <c r="D69">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E69">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F69">
         <v>17</v>
       </c>
       <c r="G69" s="1">
-        <v>59.52</v>
+        <v>58.54</v>
       </c>
       <c r="H69" s="1">
-        <v>40.48</v>
+        <v>41.46</v>
       </c>
       <c r="I69" s="2">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="J69">
         <v>0</v>
@@ -17955,19 +17955,19 @@
         <v>125</v>
       </c>
       <c r="D89">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E89">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F89">
         <v>14</v>
       </c>
       <c r="G89" s="1">
-        <v>65.84999999999999</v>
+        <v>66.67</v>
       </c>
       <c r="H89" s="1">
-        <v>34.15</v>
+        <v>33.33</v>
       </c>
       <c r="I89" s="2">
         <v>6.6</v>
@@ -18375,19 +18375,19 @@
         <v>119</v>
       </c>
       <c r="D101">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E101">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F101">
         <v>7</v>
       </c>
       <c r="G101" s="1">
-        <v>82.93000000000001</v>
+        <v>83.33</v>
       </c>
       <c r="H101" s="1">
-        <v>17.07</v>
+        <v>16.67</v>
       </c>
       <c r="I101" s="2">
         <v>7.5</v>
@@ -19005,19 +19005,19 @@
         <v>125</v>
       </c>
       <c r="D119">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E119">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F119">
         <v>8</v>
       </c>
       <c r="G119" s="1">
-        <v>80.48999999999999</v>
+        <v>80</v>
       </c>
       <c r="H119" s="1">
-        <v>19.51</v>
+        <v>20</v>
       </c>
       <c r="I119" s="2">
         <v>7</v>
@@ -19845,22 +19845,22 @@
         <v>122</v>
       </c>
       <c r="D143">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E143">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F143">
         <v>3</v>
       </c>
       <c r="G143" s="1">
-        <v>92.86</v>
+        <v>92.68000000000001</v>
       </c>
       <c r="H143" s="1">
-        <v>7.14</v>
+        <v>7.32</v>
       </c>
       <c r="I143" s="2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J143">
         <v>0</v>
@@ -20405,19 +20405,19 @@
         <v>119</v>
       </c>
       <c r="D159">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E159">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F159">
         <v>13</v>
       </c>
       <c r="G159" s="1">
-        <v>69.77</v>
+        <v>69.05</v>
       </c>
       <c r="H159" s="1">
-        <v>30.23</v>
+        <v>30.95</v>
       </c>
       <c r="I159" s="2">
         <v>6.9</v>
@@ -20790,22 +20790,22 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E170">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F170">
         <v>9</v>
       </c>
       <c r="G170" s="1">
-        <v>78.05</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="H170" s="1">
-        <v>21.95</v>
+        <v>21.43</v>
       </c>
       <c r="I170" s="2">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="J170">
         <v>0</v>
@@ -21000,22 +21000,22 @@
         <v>122</v>
       </c>
       <c r="D176">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E176">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F176">
         <v>3</v>
       </c>
       <c r="G176" s="1">
-        <v>92.68000000000001</v>
+        <v>92.86</v>
       </c>
       <c r="H176" s="1">
-        <v>7.32</v>
+        <v>7.14</v>
       </c>
       <c r="I176" s="2">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="J176">
         <v>0</v>

</xml_diff>

<commit_message>
Segundo Parcial 17 mayo tarde
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -4389,13 +4389,13 @@
         <v>30</v>
       </c>
       <c r="E104">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F104">
         <v>1</v>
       </c>
       <c r="G104" s="1">
-        <v>93.3</v>
+        <v>96.7</v>
       </c>
       <c r="H104" s="1">
         <v>3.3</v>
@@ -4404,10 +4404,10 @@
         <v>6.1</v>
       </c>
       <c r="J104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K104" s="1">
-        <v>3.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -4421,13 +4421,13 @@
         <v>208</v>
       </c>
       <c r="E105">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F105">
         <v>28</v>
       </c>
       <c r="G105" s="1">
-        <v>86.09999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="H105" s="1">
         <v>13.5</v>
@@ -4436,10 +4436,10 @@
         <v>6.3</v>
       </c>
       <c r="J105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K105" s="1">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -5902,13 +5902,13 @@
         <v>33</v>
       </c>
       <c r="E148">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F148">
         <v>4</v>
       </c>
       <c r="G148" s="1">
-        <v>84.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H148" s="1">
         <v>12.1</v>
@@ -5917,10 +5917,10 @@
         <v>7.3</v>
       </c>
       <c r="J148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -5934,13 +5934,13 @@
         <v>104</v>
       </c>
       <c r="E149">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F149">
         <v>21</v>
       </c>
       <c r="G149" s="1">
-        <v>78.8</v>
+        <v>79.8</v>
       </c>
       <c r="H149" s="1">
         <v>20.2</v>
@@ -5949,10 +5949,10 @@
         <v>7.1</v>
       </c>
       <c r="J149">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -7590,13 +7590,13 @@
         <v>36</v>
       </c>
       <c r="E197">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F197">
         <v>6</v>
       </c>
       <c r="G197" s="1">
-        <v>80.59999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H197" s="1">
         <v>16.7</v>
@@ -7605,10 +7605,10 @@
         <v>8.1</v>
       </c>
       <c r="J197">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -7625,13 +7625,13 @@
         <v>36</v>
       </c>
       <c r="E198">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F198">
         <v>5</v>
       </c>
       <c r="G198" s="1">
-        <v>83.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H198" s="1">
         <v>13.9</v>
@@ -7640,10 +7640,10 @@
         <v>7.6</v>
       </c>
       <c r="J198">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -7657,13 +7657,13 @@
         <v>114</v>
       </c>
       <c r="E199">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F199">
         <v>24</v>
       </c>
       <c r="G199" s="1">
-        <v>77.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="H199" s="1">
         <v>21.1</v>
@@ -7672,10 +7672,10 @@
         <v>7.5</v>
       </c>
       <c r="J199">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>1.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">
@@ -9307,13 +9307,13 @@
         <v>34</v>
       </c>
       <c r="E247">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F247">
         <v>11</v>
       </c>
       <c r="G247" s="1">
-        <v>64.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="H247" s="1">
         <v>32.4</v>
@@ -9322,10 +9322,10 @@
         <v>6.8</v>
       </c>
       <c r="J247">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K247" s="1">
-        <v>2.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -9409,13 +9409,13 @@
         <v>152</v>
       </c>
       <c r="E250">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F250">
         <v>81</v>
       </c>
       <c r="G250" s="1">
-        <v>45.4</v>
+        <v>46.1</v>
       </c>
       <c r="H250" s="1">
         <v>53.3</v>
@@ -9424,10 +9424,10 @@
         <v>5.6</v>
       </c>
       <c r="J250">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K250" s="1">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:11">
@@ -10767,25 +10767,25 @@
         <v>40</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F29">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="G29" s="1">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H29" s="1">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I29" s="2">
-        <v>0</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J29">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K29" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -10802,25 +10802,25 @@
         <v>38</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F30">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="G30" s="1">
-        <v>0</v>
+        <v>86.8</v>
       </c>
       <c r="H30" s="1">
-        <v>100</v>
+        <v>13.2</v>
       </c>
       <c r="I30" s="2">
-        <v>0</v>
+        <v>8.9</v>
       </c>
       <c r="J30">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="K30" s="1">
-        <v>100</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -10869,25 +10869,25 @@
         <v>114</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="F32">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="G32" s="1">
-        <v>0</v>
+        <v>62.3</v>
       </c>
       <c r="H32" s="1">
-        <v>100</v>
+        <v>37.7</v>
       </c>
       <c r="I32" s="2">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="J32">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="K32" s="1">
-        <v>100</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -12143,25 +12143,25 @@
         <v>43</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F69">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="G69" s="1">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="H69" s="1">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="I69" s="2">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="J69">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -12350,25 +12350,25 @@
         <v>278</v>
       </c>
       <c r="E75">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="F75">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="G75" s="1">
-        <v>72.3</v>
+        <v>86.7</v>
       </c>
       <c r="H75" s="1">
-        <v>27.7</v>
+        <v>13.3</v>
       </c>
       <c r="I75" s="2">
-        <v>6</v>
+        <v>7.1</v>
       </c>
       <c r="J75">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K75" s="1">
-        <v>15.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -13353,25 +13353,25 @@
         <v>30</v>
       </c>
       <c r="E104">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F104">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G104" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H104" s="1">
-        <v>96.7</v>
+        <v>33.3</v>
       </c>
       <c r="I104" s="2">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="J104">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K104" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -13385,25 +13385,25 @@
         <v>208</v>
       </c>
       <c r="E105">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="F105">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="G105" s="1">
-        <v>51</v>
+        <v>60.6</v>
       </c>
       <c r="H105" s="1">
-        <v>48.6</v>
+        <v>39.4</v>
       </c>
       <c r="I105" s="2">
-        <v>4.9</v>
+        <v>6</v>
       </c>
       <c r="J105">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="K105" s="1">
-        <v>29.8</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -13420,25 +13420,25 @@
         <v>34</v>
       </c>
       <c r="E106">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F106">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="G106" s="1">
-        <v>0</v>
+        <v>88.2</v>
       </c>
       <c r="H106" s="1">
-        <v>100</v>
+        <v>11.8</v>
       </c>
       <c r="I106" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J106">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K106" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -13455,25 +13455,25 @@
         <v>28</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F107">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="G107" s="1">
-        <v>0</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H107" s="1">
-        <v>100</v>
+        <v>3.6</v>
       </c>
       <c r="I107" s="2">
-        <v>0</v>
+        <v>7.9</v>
       </c>
       <c r="J107">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K107" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -13487,25 +13487,25 @@
         <v>62</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="F108">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="G108" s="1">
-        <v>0</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H108" s="1">
-        <v>100</v>
+        <v>8.1</v>
       </c>
       <c r="I108" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J108">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -13831,25 +13831,25 @@
         <v>31</v>
       </c>
       <c r="E118">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F118">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="G118" s="1">
-        <v>0</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="H118" s="1">
-        <v>100</v>
+        <v>19.4</v>
       </c>
       <c r="I118" s="2">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J118">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="K118" s="1">
-        <v>100</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="119" spans="1:11">
@@ -14038,25 +14038,25 @@
         <v>180</v>
       </c>
       <c r="E124">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="F124">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="G124" s="1">
-        <v>60</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="H124" s="1">
-        <v>40</v>
+        <v>26.1</v>
       </c>
       <c r="I124" s="2">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="J124">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="K124" s="1">
-        <v>34.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="125" spans="1:11">
@@ -14796,25 +14796,25 @@
         <v>31</v>
       </c>
       <c r="E146">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F146">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="G146" s="1">
-        <v>0</v>
+        <v>58.1</v>
       </c>
       <c r="H146" s="1">
-        <v>100</v>
+        <v>41.9</v>
       </c>
       <c r="I146" s="2">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="J146">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K146" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147" spans="1:11">
@@ -14831,25 +14831,25 @@
         <v>40</v>
       </c>
       <c r="E147">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F147">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="G147" s="1">
-        <v>0</v>
+        <v>77.5</v>
       </c>
       <c r="H147" s="1">
-        <v>100</v>
+        <v>22.5</v>
       </c>
       <c r="I147" s="2">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="J147">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K147" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:11">
@@ -14866,25 +14866,25 @@
         <v>33</v>
       </c>
       <c r="E148">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F148">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="G148" s="1">
-        <v>0</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H148" s="1">
-        <v>97</v>
+        <v>12.1</v>
       </c>
       <c r="I148" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J148">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -14898,25 +14898,25 @@
         <v>104</v>
       </c>
       <c r="E149">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="F149">
-        <v>103</v>
+        <v>26</v>
       </c>
       <c r="G149" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H149" s="1">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="I149" s="2">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="J149">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -15277,25 +15277,25 @@
         <v>39</v>
       </c>
       <c r="E160">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F160">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="G160" s="1">
-        <v>0</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H160" s="1">
-        <v>100</v>
+        <v>5.1</v>
       </c>
       <c r="I160" s="2">
-        <v>0</v>
+        <v>7.9</v>
       </c>
       <c r="J160">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K160" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -15379,25 +15379,25 @@
         <v>159</v>
       </c>
       <c r="E163">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="F163">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G163" s="1">
-        <v>67.90000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="H163" s="1">
-        <v>32.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I163" s="2">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
       <c r="J163">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K163" s="1">
-        <v>24.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:11">
@@ -16519,25 +16519,25 @@
         <v>42</v>
       </c>
       <c r="E196">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F196">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="G196" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H196" s="1">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="I196" s="2">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="J196">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="K196" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197" spans="1:11">
@@ -16554,25 +16554,25 @@
         <v>36</v>
       </c>
       <c r="E197">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F197">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="G197" s="1">
-        <v>0</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H197" s="1">
-        <v>97.2</v>
+        <v>11.1</v>
       </c>
       <c r="I197" s="2">
-        <v>0</v>
+        <v>8.6</v>
       </c>
       <c r="J197">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -16589,25 +16589,25 @@
         <v>36</v>
       </c>
       <c r="E198">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F198">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="G198" s="1">
-        <v>0</v>
+        <v>91.7</v>
       </c>
       <c r="H198" s="1">
-        <v>97.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I198" s="2">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="J198">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -16621,25 +16621,25 @@
         <v>114</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="F199">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="G199" s="1">
-        <v>0</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H199" s="1">
-        <v>98.2</v>
+        <v>18.4</v>
       </c>
       <c r="I199" s="2">
-        <v>0</v>
+        <v>8.1</v>
       </c>
       <c r="J199">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">
@@ -17994,25 +17994,25 @@
         <v>30</v>
       </c>
       <c r="E239">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F239">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G239" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H239" s="1">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="I239" s="2">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="J239">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K239" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="240" spans="1:11">
@@ -18029,25 +18029,25 @@
         <v>34</v>
       </c>
       <c r="E240">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F240">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G240" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H240" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I240" s="2">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J240">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K240" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241" spans="1:11">
@@ -18099,25 +18099,25 @@
         <v>28</v>
       </c>
       <c r="E242">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F242">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="G242" s="1">
-        <v>0</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H242" s="1">
-        <v>100</v>
+        <v>28.6</v>
       </c>
       <c r="I242" s="2">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="J242">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K242" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="243" spans="1:11">
@@ -18134,25 +18134,25 @@
         <v>28</v>
       </c>
       <c r="E243">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F243">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="G243" s="1">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H243" s="1">
-        <v>100</v>
+        <v>7.1</v>
       </c>
       <c r="I243" s="2">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="J243">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K243" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="244" spans="1:11">
@@ -18166,25 +18166,25 @@
         <v>172</v>
       </c>
       <c r="E244">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="F244">
-        <v>172</v>
+        <v>68</v>
       </c>
       <c r="G244" s="1">
-        <v>0</v>
+        <v>60.5</v>
       </c>
       <c r="H244" s="1">
-        <v>100</v>
+        <v>39.5</v>
       </c>
       <c r="I244" s="2">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="J244">
-        <v>172</v>
+        <v>52</v>
       </c>
       <c r="K244" s="1">
-        <v>100</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="245" spans="1:11">
@@ -18201,25 +18201,25 @@
         <v>30</v>
       </c>
       <c r="E245">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F245">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="G245" s="1">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="H245" s="1">
-        <v>96.7</v>
+        <v>63.3</v>
       </c>
       <c r="I245" s="2">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="J245">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K245" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246" spans="1:11">
@@ -18236,25 +18236,25 @@
         <v>30</v>
       </c>
       <c r="E246">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F246">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="G246" s="1">
-        <v>0</v>
+        <v>36.7</v>
       </c>
       <c r="H246" s="1">
-        <v>100</v>
+        <v>63.3</v>
       </c>
       <c r="I246" s="2">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="J246">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K246" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:11">
@@ -18271,25 +18271,25 @@
         <v>34</v>
       </c>
       <c r="E247">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F247">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="G247" s="1">
-        <v>0</v>
+        <v>76.5</v>
       </c>
       <c r="H247" s="1">
-        <v>97.09999999999999</v>
+        <v>23.5</v>
       </c>
       <c r="I247" s="2">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="J247">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K247" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -18306,25 +18306,25 @@
         <v>33</v>
       </c>
       <c r="E248">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F248">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G248" s="1">
-        <v>0</v>
+        <v>63.6</v>
       </c>
       <c r="H248" s="1">
-        <v>100</v>
+        <v>36.4</v>
       </c>
       <c r="I248" s="2">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="J248">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K248" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:11">
@@ -18341,25 +18341,25 @@
         <v>25</v>
       </c>
       <c r="E249">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F249">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G249" s="1">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H249" s="1">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="I249" s="2">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="J249">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K249" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:11">
@@ -18373,25 +18373,25 @@
         <v>152</v>
       </c>
       <c r="E250">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="F250">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="G250" s="1">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H250" s="1">
-        <v>98.7</v>
+        <v>49.3</v>
       </c>
       <c r="I250" s="2">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="J250">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="K250" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:11">
@@ -19743,7 +19743,7 @@
         <v>5</v>
       </c>
       <c r="I29" s="2">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="J29">
         <v>40</v>
@@ -19766,16 +19766,16 @@
         <v>38</v>
       </c>
       <c r="E30">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F30">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G30" s="1">
-        <v>94.7</v>
+        <v>89.5</v>
       </c>
       <c r="H30" s="1">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="I30" s="2">
         <v>9.199999999999999</v>
@@ -19833,19 +19833,19 @@
         <v>114</v>
       </c>
       <c r="E32">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F32">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G32" s="1">
-        <v>96.5</v>
+        <v>94.7</v>
       </c>
       <c r="H32" s="1">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="I32" s="2">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="J32">
         <v>114</v>
@@ -21119,7 +21119,7 @@
         <v>7</v>
       </c>
       <c r="I69" s="2">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J69">
         <v>43</v>
@@ -22317,19 +22317,19 @@
         <v>30</v>
       </c>
       <c r="E104">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F104">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G104" s="1">
-        <v>93.3</v>
+        <v>66.7</v>
       </c>
       <c r="H104" s="1">
-        <v>3.3</v>
+        <v>33.3</v>
       </c>
       <c r="I104" s="2">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="J104">
         <v>30</v>
@@ -22349,19 +22349,19 @@
         <v>208</v>
       </c>
       <c r="E105">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="F105">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="G105" s="1">
-        <v>79.8</v>
+        <v>76</v>
       </c>
       <c r="H105" s="1">
-        <v>19.7</v>
+        <v>24</v>
       </c>
       <c r="I105" s="2">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="J105">
         <v>208</v>
@@ -22384,19 +22384,19 @@
         <v>34</v>
       </c>
       <c r="E106">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F106">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G106" s="1">
-        <v>94.09999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="H106" s="1">
-        <v>5.9</v>
+        <v>11.8</v>
       </c>
       <c r="I106" s="2">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J106">
         <v>34</v>
@@ -22431,7 +22431,7 @@
         <v>3.6</v>
       </c>
       <c r="I107" s="2">
-        <v>9.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J107">
         <v>28</v>
@@ -22451,19 +22451,19 @@
         <v>62</v>
       </c>
       <c r="E108">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F108">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G108" s="1">
-        <v>95.2</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H108" s="1">
-        <v>4.8</v>
+        <v>8.1</v>
       </c>
       <c r="I108" s="2">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J108">
         <v>62</v>
@@ -22795,19 +22795,19 @@
         <v>31</v>
       </c>
       <c r="E118">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F118">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G118" s="1">
-        <v>74.2</v>
+        <v>93.5</v>
       </c>
       <c r="H118" s="1">
-        <v>25.8</v>
+        <v>6.5</v>
       </c>
       <c r="I118" s="2">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="J118">
         <v>31</v>
@@ -23002,19 +23002,19 @@
         <v>180</v>
       </c>
       <c r="E124">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F124">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G124" s="1">
-        <v>90</v>
+        <v>93.3</v>
       </c>
       <c r="H124" s="1">
-        <v>10</v>
+        <v>6.7</v>
       </c>
       <c r="I124" s="2">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="J124">
         <v>180</v>
@@ -23760,19 +23760,19 @@
         <v>31</v>
       </c>
       <c r="E146">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F146">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G146" s="1">
-        <v>71</v>
+        <v>58.1</v>
       </c>
       <c r="H146" s="1">
-        <v>29</v>
+        <v>41.9</v>
       </c>
       <c r="I146" s="2">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="J146">
         <v>31</v>
@@ -23795,19 +23795,19 @@
         <v>40</v>
       </c>
       <c r="E147">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F147">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G147" s="1">
-        <v>80</v>
+        <v>77.5</v>
       </c>
       <c r="H147" s="1">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="I147" s="2">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="J147">
         <v>40</v>
@@ -23830,19 +23830,19 @@
         <v>33</v>
       </c>
       <c r="E148">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F148">
         <v>4</v>
       </c>
       <c r="G148" s="1">
-        <v>84.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H148" s="1">
         <v>12.1</v>
       </c>
       <c r="I148" s="2">
-        <v>7.3</v>
+        <v>7.7</v>
       </c>
       <c r="J148">
         <v>33</v>
@@ -23862,19 +23862,19 @@
         <v>104</v>
       </c>
       <c r="E149">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F149">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G149" s="1">
-        <v>78.8</v>
+        <v>75</v>
       </c>
       <c r="H149" s="1">
-        <v>20.2</v>
+        <v>25</v>
       </c>
       <c r="I149" s="2">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="J149">
         <v>104</v>
@@ -24253,7 +24253,7 @@
         <v>5.1</v>
       </c>
       <c r="I160" s="2">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="J160">
         <v>39</v>
@@ -25483,16 +25483,16 @@
         <v>42</v>
       </c>
       <c r="E196">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F196">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G196" s="1">
-        <v>69</v>
+        <v>66.7</v>
       </c>
       <c r="H196" s="1">
-        <v>31</v>
+        <v>33.3</v>
       </c>
       <c r="I196" s="2">
         <v>6.9</v>
@@ -25518,19 +25518,19 @@
         <v>36</v>
       </c>
       <c r="E197">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F197">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G197" s="1">
-        <v>80.59999999999999</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H197" s="1">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="I197" s="2">
-        <v>8.1</v>
+        <v>8.5</v>
       </c>
       <c r="J197">
         <v>36</v>
@@ -25553,19 +25553,19 @@
         <v>36</v>
       </c>
       <c r="E198">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F198">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G198" s="1">
-        <v>83.3</v>
+        <v>91.7</v>
       </c>
       <c r="H198" s="1">
-        <v>13.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I198" s="2">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J198">
         <v>36</v>
@@ -25585,19 +25585,19 @@
         <v>114</v>
       </c>
       <c r="E199">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F199">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G199" s="1">
-        <v>77.2</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H199" s="1">
-        <v>21.1</v>
+        <v>18.4</v>
       </c>
       <c r="I199" s="2">
-        <v>7.5</v>
+        <v>7.9</v>
       </c>
       <c r="J199">
         <v>114</v>
@@ -26958,19 +26958,19 @@
         <v>30</v>
       </c>
       <c r="E239">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F239">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G239" s="1">
-        <v>76.7</v>
+        <v>80</v>
       </c>
       <c r="H239" s="1">
-        <v>23.3</v>
+        <v>20</v>
       </c>
       <c r="I239" s="2">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="J239">
         <v>30</v>
@@ -26993,19 +26993,19 @@
         <v>34</v>
       </c>
       <c r="E240">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F240">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G240" s="1">
-        <v>91.2</v>
+        <v>100</v>
       </c>
       <c r="H240" s="1">
-        <v>8.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="I240" s="2">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J240">
         <v>34</v>
@@ -27098,19 +27098,19 @@
         <v>28</v>
       </c>
       <c r="E243">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F243">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G243" s="1">
-        <v>89.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H243" s="1">
-        <v>10.7</v>
+        <v>7.1</v>
       </c>
       <c r="I243" s="2">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="J243">
         <v>28</v>
@@ -27130,19 +27130,19 @@
         <v>172</v>
       </c>
       <c r="E244">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F244">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G244" s="1">
-        <v>82</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="H244" s="1">
-        <v>18</v>
+        <v>15.1</v>
       </c>
       <c r="I244" s="2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="J244">
         <v>172</v>
@@ -27165,19 +27165,19 @@
         <v>30</v>
       </c>
       <c r="E245">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F245">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G245" s="1">
-        <v>30</v>
+        <v>33.3</v>
       </c>
       <c r="H245" s="1">
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="I245" s="2">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="J245">
         <v>30</v>
@@ -27212,7 +27212,7 @@
         <v>63.3</v>
       </c>
       <c r="I246" s="2">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="J246">
         <v>30</v>
@@ -27235,19 +27235,19 @@
         <v>34</v>
       </c>
       <c r="E247">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F247">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G247" s="1">
-        <v>64.7</v>
+        <v>76.5</v>
       </c>
       <c r="H247" s="1">
-        <v>32.4</v>
+        <v>23.5</v>
       </c>
       <c r="I247" s="2">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="J247">
         <v>34</v>
@@ -27270,19 +27270,19 @@
         <v>33</v>
       </c>
       <c r="E248">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F248">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G248" s="1">
-        <v>54.5</v>
+        <v>63.6</v>
       </c>
       <c r="H248" s="1">
-        <v>45.5</v>
+        <v>36.4</v>
       </c>
       <c r="I248" s="2">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="J248">
         <v>33</v>
@@ -27305,16 +27305,16 @@
         <v>25</v>
       </c>
       <c r="E249">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F249">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G249" s="1">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H249" s="1">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I249" s="2">
         <v>6.1</v>
@@ -27337,19 +27337,19 @@
         <v>152</v>
       </c>
       <c r="E250">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="F250">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G250" s="1">
-        <v>45.4</v>
+        <v>50</v>
       </c>
       <c r="H250" s="1">
-        <v>53.9</v>
+        <v>50</v>
       </c>
       <c r="I250" s="2">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="J250">
         <v>152</v>

</xml_diff>

<commit_message>
Segundo Parcial 17 mayo tarde2
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -11350,25 +11350,25 @@
         <v>27</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F46">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="G46" s="1">
-        <v>0</v>
+        <v>59.3</v>
       </c>
       <c r="H46" s="1">
-        <v>100</v>
+        <v>40.7</v>
       </c>
       <c r="I46" s="2">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="J46">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K46" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -11420,25 +11420,25 @@
         <v>26</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F48">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="G48" s="1">
-        <v>0</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H48" s="1">
-        <v>100</v>
+        <v>26.9</v>
       </c>
       <c r="I48" s="2">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="J48">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="K48" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -11455,25 +11455,25 @@
         <v>17</v>
       </c>
       <c r="E49">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F49">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
-        <v>70.59999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H49" s="1">
-        <v>29.4</v>
+        <v>5.9</v>
       </c>
       <c r="I49" s="2">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="J49">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>23.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -11522,25 +11522,25 @@
         <v>119</v>
       </c>
       <c r="E51">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="F51">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="G51" s="1">
-        <v>34.5</v>
+        <v>67.2</v>
       </c>
       <c r="H51" s="1">
-        <v>65.5</v>
+        <v>32.8</v>
       </c>
       <c r="I51" s="2">
-        <v>4.1</v>
+        <v>6.8</v>
       </c>
       <c r="J51">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="K51" s="1">
-        <v>47.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -12936,25 +12936,25 @@
         <v>30</v>
       </c>
       <c r="E92">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F92">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="G92" s="1">
-        <v>0</v>
+        <v>86.7</v>
       </c>
       <c r="H92" s="1">
-        <v>96.7</v>
+        <v>10</v>
       </c>
       <c r="I92" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J92">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K92" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:11">
@@ -12971,25 +12971,25 @@
         <v>31</v>
       </c>
       <c r="E93">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F93">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G93" s="1">
-        <v>0</v>
+        <v>58.1</v>
       </c>
       <c r="H93" s="1">
-        <v>87.09999999999999</v>
+        <v>38.7</v>
       </c>
       <c r="I93" s="2">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="J93">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K93" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:11">
@@ -13006,25 +13006,25 @@
         <v>34</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F94">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="G94" s="1">
-        <v>0</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H94" s="1">
-        <v>94.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="I94" s="2">
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="J94">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="K94" s="1">
-        <v>100</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -13041,25 +13041,25 @@
         <v>25</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F95">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G95" s="1">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="H95" s="1">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="I95" s="2">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="J95">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="K95" s="1">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row r="96" spans="1:11">
@@ -13076,25 +13076,25 @@
         <v>29</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F96">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="G96" s="1">
-        <v>0</v>
+        <v>82.8</v>
       </c>
       <c r="H96" s="1">
-        <v>96.59999999999999</v>
+        <v>13.8</v>
       </c>
       <c r="I96" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J96">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="K96" s="1">
-        <v>100</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="97" spans="1:11">
@@ -13111,25 +13111,25 @@
         <v>14</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F97">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G97" s="1">
-        <v>0</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H97" s="1">
-        <v>100</v>
+        <v>7.1</v>
       </c>
       <c r="I97" s="2">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="J97">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K97" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:11">
@@ -13143,25 +13143,25 @@
         <v>163</v>
       </c>
       <c r="E98">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="F98">
-        <v>154</v>
+        <v>33</v>
       </c>
       <c r="G98" s="1">
-        <v>0</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="H98" s="1">
-        <v>94.5</v>
+        <v>20.2</v>
       </c>
       <c r="I98" s="2">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="J98">
-        <v>163</v>
+        <v>15</v>
       </c>
       <c r="K98" s="1">
-        <v>100</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="99" spans="1:11">
@@ -13318,25 +13318,25 @@
         <v>32</v>
       </c>
       <c r="E103">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F103">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="G103" s="1">
-        <v>0</v>
+        <v>56.2</v>
       </c>
       <c r="H103" s="1">
-        <v>100</v>
+        <v>43.8</v>
       </c>
       <c r="I103" s="2">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="J103">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K103" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:11">
@@ -13385,25 +13385,25 @@
         <v>208</v>
       </c>
       <c r="E105">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="F105">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="G105" s="1">
-        <v>60.6</v>
+        <v>69.2</v>
       </c>
       <c r="H105" s="1">
-        <v>39.4</v>
+        <v>30.8</v>
       </c>
       <c r="I105" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J105">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K105" s="1">
-        <v>15.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -14554,25 +14554,25 @@
         <v>31</v>
       </c>
       <c r="E139">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F139">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G139" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H139" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I139" s="2">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="J139">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K139" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:11">
@@ -14589,25 +14589,25 @@
         <v>27</v>
       </c>
       <c r="E140">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F140">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G140" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H140" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I140" s="2">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="J140">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K140" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:11">
@@ -14624,25 +14624,25 @@
         <v>41</v>
       </c>
       <c r="E141">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F141">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="G141" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H141" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I141" s="2">
-        <v>0</v>
+        <v>8.1</v>
       </c>
       <c r="J141">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K141" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:11">
@@ -14659,25 +14659,25 @@
         <v>30</v>
       </c>
       <c r="E142">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F142">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G142" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H142" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I142" s="2">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="J142">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K142" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:11">
@@ -14694,25 +14694,25 @@
         <v>20</v>
       </c>
       <c r="E143">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F143">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G143" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H143" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I143" s="2">
-        <v>0</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J143">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -14729,25 +14729,25 @@
         <v>28</v>
       </c>
       <c r="E144">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F144">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G144" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H144" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I144" s="2">
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="J144">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K144" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145" spans="1:11">
@@ -14761,25 +14761,25 @@
         <v>177</v>
       </c>
       <c r="E145">
-        <v>0</v>
+        <v>177</v>
       </c>
       <c r="F145">
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="G145" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H145" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I145" s="2">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="J145">
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="K145" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -15863,25 +15863,25 @@
         <v>41</v>
       </c>
       <c r="E177">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F177">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="G177" s="1">
-        <v>0</v>
+        <v>92.7</v>
       </c>
       <c r="H177" s="1">
-        <v>100</v>
+        <v>7.3</v>
       </c>
       <c r="I177" s="2">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="J177">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K177" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:11">
@@ -15910,13 +15910,13 @@
         <v>36.7</v>
       </c>
       <c r="I178" s="2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J178">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K178" s="1">
-        <v>3.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179" spans="1:11">
@@ -15933,25 +15933,25 @@
         <v>33</v>
       </c>
       <c r="E179">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F179">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G179" s="1">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="H179" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I179" s="2">
         <v>7.9</v>
       </c>
       <c r="J179">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K179" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:11">
@@ -16070,25 +16070,25 @@
         <v>226</v>
       </c>
       <c r="E183">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="F183">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="G183" s="1">
-        <v>73.90000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="H183" s="1">
-        <v>26.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I183" s="2">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="J183">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -17344,25 +17344,25 @@
         <v>33</v>
       </c>
       <c r="E220">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F220">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="G220" s="1">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H220" s="1">
-        <v>100</v>
+        <v>9.1</v>
       </c>
       <c r="I220" s="2">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J220">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K220" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221" spans="1:11">
@@ -17376,25 +17376,25 @@
         <v>33</v>
       </c>
       <c r="E221">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F221">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="G221" s="1">
-        <v>0</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H221" s="1">
-        <v>100</v>
+        <v>9.1</v>
       </c>
       <c r="I221" s="2">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J221">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K221" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222" spans="1:11">
@@ -18064,25 +18064,25 @@
         <v>20</v>
       </c>
       <c r="E241">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F241">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G241" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H241" s="1">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I241" s="2">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="J241">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K241" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="242" spans="1:11">
@@ -18166,25 +18166,25 @@
         <v>172</v>
       </c>
       <c r="E244">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="F244">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="G244" s="1">
-        <v>60.5</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="H244" s="1">
-        <v>39.5</v>
+        <v>29.1</v>
       </c>
       <c r="I244" s="2">
-        <v>4.9</v>
+        <v>6</v>
       </c>
       <c r="J244">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="K244" s="1">
-        <v>30.2</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="245" spans="1:11">
@@ -20314,19 +20314,19 @@
         <v>27</v>
       </c>
       <c r="E46">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G46" s="1">
-        <v>66.7</v>
+        <v>59.3</v>
       </c>
       <c r="H46" s="1">
-        <v>33.3</v>
+        <v>40.7</v>
       </c>
       <c r="I46" s="2">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="J46">
         <v>27</v>
@@ -20384,19 +20384,19 @@
         <v>26</v>
       </c>
       <c r="E48">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F48">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G48" s="1">
-        <v>88.5</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H48" s="1">
-        <v>11.5</v>
+        <v>26.9</v>
       </c>
       <c r="I48" s="2">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="J48">
         <v>26</v>
@@ -20486,16 +20486,16 @@
         <v>119</v>
       </c>
       <c r="E51">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F51">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G51" s="1">
-        <v>72.3</v>
+        <v>67.2</v>
       </c>
       <c r="H51" s="1">
-        <v>27.7</v>
+        <v>32.8</v>
       </c>
       <c r="I51" s="2">
         <v>7</v>
@@ -21900,19 +21900,19 @@
         <v>30</v>
       </c>
       <c r="E92">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F92">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G92" s="1">
-        <v>93.3</v>
+        <v>86.7</v>
       </c>
       <c r="H92" s="1">
-        <v>6.7</v>
+        <v>13.3</v>
       </c>
       <c r="I92" s="2">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="J92">
         <v>30</v>
@@ -21935,19 +21935,19 @@
         <v>31</v>
       </c>
       <c r="E93">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F93">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G93" s="1">
-        <v>61.3</v>
+        <v>58.1</v>
       </c>
       <c r="H93" s="1">
-        <v>38.7</v>
+        <v>41.9</v>
       </c>
       <c r="I93" s="2">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="J93">
         <v>31</v>
@@ -21970,19 +21970,19 @@
         <v>34</v>
       </c>
       <c r="E94">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F94">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G94" s="1">
-        <v>88.2</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H94" s="1">
-        <v>8.800000000000001</v>
+        <v>2.9</v>
       </c>
       <c r="I94" s="2">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="J94">
         <v>34</v>
@@ -22017,7 +22017,7 @@
         <v>40</v>
       </c>
       <c r="I95" s="2">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="J95">
         <v>25</v>
@@ -22040,19 +22040,19 @@
         <v>29</v>
       </c>
       <c r="E96">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F96">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G96" s="1">
-        <v>86.2</v>
+        <v>82.8</v>
       </c>
       <c r="H96" s="1">
-        <v>10.3</v>
+        <v>13.8</v>
       </c>
       <c r="I96" s="2">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="J96">
         <v>29</v>
@@ -22075,19 +22075,19 @@
         <v>14</v>
       </c>
       <c r="E97">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" s="1">
-        <v>100</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H97" s="1">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="I97" s="2">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="J97">
         <v>14</v>
@@ -22107,19 +22107,19 @@
         <v>163</v>
       </c>
       <c r="E98">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F98">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G98" s="1">
-        <v>80.40000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="H98" s="1">
-        <v>18.4</v>
+        <v>20.2</v>
       </c>
       <c r="I98" s="2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="J98">
         <v>163</v>
@@ -22282,19 +22282,19 @@
         <v>32</v>
       </c>
       <c r="E103">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F103">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G103" s="1">
-        <v>100</v>
+        <v>56.2</v>
       </c>
       <c r="H103" s="1">
-        <v>0</v>
+        <v>43.8</v>
       </c>
       <c r="I103" s="2">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="J103">
         <v>32</v>
@@ -22349,16 +22349,16 @@
         <v>208</v>
       </c>
       <c r="E105">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="F105">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G105" s="1">
-        <v>76</v>
+        <v>69.2</v>
       </c>
       <c r="H105" s="1">
-        <v>24</v>
+        <v>30.8</v>
       </c>
       <c r="I105" s="2">
         <v>6.8</v>
@@ -23530,7 +23530,7 @@
         <v>0</v>
       </c>
       <c r="I139" s="2">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="J139">
         <v>31</v>
@@ -23565,7 +23565,7 @@
         <v>0</v>
       </c>
       <c r="I140" s="2">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="J140">
         <v>27</v>
@@ -23635,7 +23635,7 @@
         <v>0</v>
       </c>
       <c r="I142" s="2">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="J142">
         <v>30</v>
@@ -23670,7 +23670,7 @@
         <v>0</v>
       </c>
       <c r="I143" s="2">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J143">
         <v>20</v>
@@ -23705,7 +23705,7 @@
         <v>0</v>
       </c>
       <c r="I144" s="2">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="J144">
         <v>28</v>
@@ -23737,7 +23737,7 @@
         <v>0</v>
       </c>
       <c r="I145" s="2">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="J145">
         <v>177</v>
@@ -24839,7 +24839,7 @@
         <v>7.3</v>
       </c>
       <c r="I177" s="2">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="J177">
         <v>41</v>
@@ -25046,7 +25046,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I183" s="2">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="J183">
         <v>226</v>
@@ -26308,19 +26308,19 @@
         <v>33</v>
       </c>
       <c r="E220">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F220">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G220" s="1">
-        <v>93.90000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H220" s="1">
-        <v>6.1</v>
+        <v>9.1</v>
       </c>
       <c r="I220" s="2">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="J220">
         <v>33</v>
@@ -26340,19 +26340,19 @@
         <v>33</v>
       </c>
       <c r="E221">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F221">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G221" s="1">
-        <v>93.90000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H221" s="1">
-        <v>6.1</v>
+        <v>9.1</v>
       </c>
       <c r="I221" s="2">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="J221">
         <v>33</v>

</xml_diff>

<commit_message>
Finales Lunes Tarde Noche
</commit_message>
<xml_diff>
--- a/DetalleXDocente.xlsx
+++ b/DetalleXDocente.xlsx
@@ -18976,25 +18976,25 @@
         <v>31</v>
       </c>
       <c r="E7">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G7" s="1">
-        <v>77.40000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H7" s="1">
-        <v>22.6</v>
+        <v>12.9</v>
       </c>
       <c r="I7" s="2">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="J7">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -19011,25 +19011,25 @@
         <v>41</v>
       </c>
       <c r="E8">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G8" s="1">
-        <v>82.90000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="H8" s="1">
-        <v>17.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I8" s="2">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="J8">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K8" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -19046,25 +19046,25 @@
         <v>28</v>
       </c>
       <c r="E9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="1">
-        <v>85.7</v>
+        <v>89.3</v>
       </c>
       <c r="H9" s="1">
-        <v>14.3</v>
+        <v>10.7</v>
       </c>
       <c r="I9" s="2">
         <v>8</v>
       </c>
       <c r="J9">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K9" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -19081,16 +19081,16 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10" s="1">
-        <v>86.8</v>
+        <v>84.2</v>
       </c>
       <c r="H10" s="1">
-        <v>13.2</v>
+        <v>15.8</v>
       </c>
       <c r="I10" s="2">
         <v>7.7</v>
@@ -19116,25 +19116,25 @@
         <v>28</v>
       </c>
       <c r="E11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G11" s="1">
-        <v>75</v>
+        <v>85.7</v>
       </c>
       <c r="H11" s="1">
-        <v>25</v>
+        <v>14.3</v>
       </c>
       <c r="I11" s="2">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="J11">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -19151,25 +19151,25 @@
         <v>41</v>
       </c>
       <c r="E12">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F12">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G12" s="1">
-        <v>63.4</v>
+        <v>78</v>
       </c>
       <c r="H12" s="1">
-        <v>36.6</v>
+        <v>22</v>
       </c>
       <c r="I12" s="2">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="J12">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K12" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -19183,25 +19183,25 @@
         <v>207</v>
       </c>
       <c r="E13">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="F13">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G13" s="1">
-        <v>78.3</v>
+        <v>85.5</v>
       </c>
       <c r="H13" s="1">
-        <v>21.7</v>
+        <v>14.5</v>
       </c>
       <c r="I13" s="2">
         <v>7.6</v>
       </c>
       <c r="J13">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="K13" s="1">
-        <v>81.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -19390,25 +19390,25 @@
         <v>42</v>
       </c>
       <c r="E19">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="1">
-        <v>97.59999999999999</v>
+        <v>95.2</v>
       </c>
       <c r="H19" s="1">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="I19" s="2">
-        <v>9.1</v>
+        <v>8.5</v>
       </c>
       <c r="J19">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="K19" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -19425,25 +19425,25 @@
         <v>41</v>
       </c>
       <c r="E20">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G20" s="1">
-        <v>92.7</v>
+        <v>87.8</v>
       </c>
       <c r="H20" s="1">
-        <v>7.3</v>
+        <v>12.2</v>
       </c>
       <c r="I20" s="2">
-        <v>8.699999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="J20">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -19457,25 +19457,25 @@
         <v>168</v>
       </c>
       <c r="E21">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G21" s="1">
-        <v>91.7</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="H21" s="1">
-        <v>8.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="I21" s="2">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="J21">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="K21" s="1">
-        <v>49.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -19868,25 +19868,25 @@
         <v>31</v>
       </c>
       <c r="E33">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F33">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G33" s="1">
-        <v>61.3</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="H33" s="1">
-        <v>38.7</v>
+        <v>19.4</v>
       </c>
       <c r="I33" s="2">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="J33">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K33" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -19938,25 +19938,25 @@
         <v>30</v>
       </c>
       <c r="E35">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F35">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G35" s="1">
-        <v>76.7</v>
+        <v>86.7</v>
       </c>
       <c r="H35" s="1">
-        <v>23.3</v>
+        <v>13.3</v>
       </c>
       <c r="I35" s="2">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="J35">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K35" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -19973,25 +19973,25 @@
         <v>33</v>
       </c>
       <c r="E36">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G36" s="1">
-        <v>78.8</v>
+        <v>100</v>
       </c>
       <c r="H36" s="1">
-        <v>21.2</v>
+        <v>0</v>
       </c>
       <c r="I36" s="2">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="J36">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K36" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -20008,25 +20008,25 @@
         <v>33</v>
       </c>
       <c r="E37">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F37">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G37" s="1">
-        <v>81.8</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H37" s="1">
-        <v>18.2</v>
+        <v>6.1</v>
       </c>
       <c r="I37" s="2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="J37">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K37" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -20040,25 +20040,25 @@
         <v>168</v>
       </c>
       <c r="E38">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="F38">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="G38" s="1">
-        <v>74.40000000000001</v>
+        <v>86.3</v>
       </c>
       <c r="H38" s="1">
-        <v>25.6</v>
+        <v>13.7</v>
       </c>
       <c r="I38" s="2">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="J38">
-        <v>168</v>
+        <v>41</v>
       </c>
       <c r="K38" s="1">
-        <v>100</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -20177,25 +20177,25 @@
         <v>39</v>
       </c>
       <c r="E42">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G42" s="1">
-        <v>84.59999999999999</v>
+        <v>87.2</v>
       </c>
       <c r="H42" s="1">
-        <v>15.4</v>
+        <v>12.8</v>
       </c>
       <c r="I42" s="2">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="J42">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K42" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -20247,16 +20247,16 @@
         <v>25</v>
       </c>
       <c r="E44">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F44">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G44" s="1">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H44" s="1">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I44" s="2">
         <v>6.6</v>
@@ -20279,25 +20279,25 @@
         <v>94</v>
       </c>
       <c r="E45">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F45">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G45" s="1">
-        <v>75.5</v>
+        <v>77.7</v>
       </c>
       <c r="H45" s="1">
-        <v>24.5</v>
+        <v>22.3</v>
       </c>
       <c r="I45" s="2">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="J45">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K45" s="1">
-        <v>41.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -20626,19 +20626,19 @@
         <v>21</v>
       </c>
       <c r="E55">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G55" s="1">
-        <v>85.7</v>
+        <v>90.5</v>
       </c>
       <c r="H55" s="1">
-        <v>14.3</v>
+        <v>9.5</v>
       </c>
       <c r="I55" s="2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="J55">
         <v>0</v>
@@ -20728,16 +20728,16 @@
         <v>135</v>
       </c>
       <c r="E58">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F58">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G58" s="1">
-        <v>85.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="H58" s="1">
-        <v>14.8</v>
+        <v>14.1</v>
       </c>
       <c r="I58" s="2">
         <v>6.8</v>
@@ -21623,25 +21623,25 @@
         <v>37</v>
       </c>
       <c r="E84">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F84">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G84" s="1">
-        <v>59.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="H84" s="1">
-        <v>40.5</v>
+        <v>32.4</v>
       </c>
       <c r="I84" s="2">
         <v>6.4</v>
       </c>
       <c r="J84">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K84" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -21658,25 +21658,25 @@
         <v>31</v>
       </c>
       <c r="E85">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F85">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G85" s="1">
-        <v>35.5</v>
+        <v>51.6</v>
       </c>
       <c r="H85" s="1">
-        <v>64.5</v>
+        <v>48.4</v>
       </c>
       <c r="I85" s="2">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="J85">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K85" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -21693,25 +21693,25 @@
         <v>41</v>
       </c>
       <c r="E86">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F86">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G86" s="1">
-        <v>46.3</v>
+        <v>58.5</v>
       </c>
       <c r="H86" s="1">
-        <v>53.7</v>
+        <v>41.5</v>
       </c>
       <c r="I86" s="2">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="J86">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K86" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:11">
@@ -21728,25 +21728,25 @@
         <v>31</v>
       </c>
       <c r="E87">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F87">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G87" s="1">
-        <v>54.8</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="H87" s="1">
-        <v>45.2</v>
+        <v>19.4</v>
       </c>
       <c r="I87" s="2">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="J87">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K87" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:11">
@@ -21763,25 +21763,25 @@
         <v>38</v>
       </c>
       <c r="E88">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F88">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G88" s="1">
-        <v>86.8</v>
+        <v>84.2</v>
       </c>
       <c r="H88" s="1">
-        <v>13.2</v>
+        <v>15.8</v>
       </c>
       <c r="I88" s="2">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="J88">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K88" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:11">
@@ -21798,25 +21798,25 @@
         <v>28</v>
       </c>
       <c r="E89">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F89">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G89" s="1">
-        <v>64.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="H89" s="1">
-        <v>35.7</v>
+        <v>21.4</v>
       </c>
       <c r="I89" s="2">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="J89">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K89" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:11">
@@ -21833,25 +21833,25 @@
         <v>41</v>
       </c>
       <c r="E90">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F90">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G90" s="1">
-        <v>58.5</v>
+        <v>73.2</v>
       </c>
       <c r="H90" s="1">
-        <v>41.5</v>
+        <v>26.8</v>
       </c>
       <c r="I90" s="2">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="J90">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K90" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -21865,25 +21865,25 @@
         <v>247</v>
       </c>
       <c r="E91">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="F91">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="G91" s="1">
-        <v>58.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="H91" s="1">
-        <v>41.7</v>
+        <v>29.6</v>
       </c>
       <c r="I91" s="2">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J91">
-        <v>247</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -22658,25 +22658,25 @@
         <v>39</v>
       </c>
       <c r="E114">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F114">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G114" s="1">
-        <v>56.4</v>
+        <v>87.2</v>
       </c>
       <c r="H114" s="1">
-        <v>43.6</v>
+        <v>12.8</v>
       </c>
       <c r="I114" s="2">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
       <c r="J114">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K114" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:11">
@@ -22760,25 +22760,25 @@
         <v>87</v>
       </c>
       <c r="E117">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="F117">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>79.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H117" s="1">
-        <v>20.7</v>
+        <v>6.9</v>
       </c>
       <c r="I117" s="2">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="J117">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K117" s="1">
-        <v>44.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:11">
@@ -23244,16 +23244,16 @@
         <v>31</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F131">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G131" s="1">
-        <v>96.8</v>
+        <v>100</v>
       </c>
       <c r="H131" s="1">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I131" s="2">
         <v>7.2</v>
@@ -23276,16 +23276,16 @@
         <v>61</v>
       </c>
       <c r="E132">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F132">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G132" s="1">
-        <v>88.5</v>
+        <v>90.2</v>
       </c>
       <c r="H132" s="1">
-        <v>11.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I132" s="2">
         <v>7.3</v>
@@ -24206,25 +24206,25 @@
         <v>43</v>
       </c>
       <c r="E159">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F159">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G159" s="1">
-        <v>97.7</v>
+        <v>90.7</v>
       </c>
       <c r="H159" s="1">
-        <v>2.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I159" s="2">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J159">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="K159" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:11">
@@ -24241,25 +24241,25 @@
         <v>39</v>
       </c>
       <c r="E160">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F160">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G160" s="1">
-        <v>94.90000000000001</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="H160" s="1">
-        <v>5.1</v>
+        <v>15.4</v>
       </c>
       <c r="I160" s="2">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="J160">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K160" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -24276,25 +24276,25 @@
         <v>40</v>
       </c>
       <c r="E161">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F161">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G161" s="1">
-        <v>82.5</v>
+        <v>80</v>
       </c>
       <c r="H161" s="1">
-        <v>17.5</v>
+        <v>20</v>
       </c>
       <c r="I161" s="2">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
       <c r="J161">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K161" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:11">
@@ -24311,25 +24311,25 @@
         <v>37</v>
       </c>
       <c r="E162">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F162">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G162" s="1">
-        <v>89.2</v>
+        <v>75.7</v>
       </c>
       <c r="H162" s="1">
-        <v>10.8</v>
+        <v>24.3</v>
       </c>
       <c r="I162" s="2">
-        <v>8.1</v>
+        <v>7.3</v>
       </c>
       <c r="J162">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K162" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:11">
@@ -24343,25 +24343,25 @@
         <v>159</v>
       </c>
       <c r="E163">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="F163">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G163" s="1">
-        <v>91.2</v>
+        <v>83</v>
       </c>
       <c r="H163" s="1">
-        <v>8.800000000000001</v>
+        <v>17</v>
       </c>
       <c r="I163" s="2">
-        <v>8.6</v>
+        <v>7.8</v>
       </c>
       <c r="J163">
-        <v>159</v>
+        <v>0</v>
       </c>
       <c r="K163" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:11">
@@ -24690,16 +24690,16 @@
         <v>28</v>
       </c>
       <c r="E173">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F173">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G173" s="1">
-        <v>96.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H173" s="1">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="I173" s="2">
         <v>7.6</v>
@@ -24757,16 +24757,16 @@
         <v>180</v>
       </c>
       <c r="E175">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F175">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G175" s="1">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H175" s="1">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="I175" s="2">
         <v>8.199999999999999</v>
@@ -24827,25 +24827,25 @@
         <v>41</v>
       </c>
       <c r="E177">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F177">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G177" s="1">
-        <v>92.7</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="H177" s="1">
-        <v>7.3</v>
+        <v>2.4</v>
       </c>
       <c r="I177" s="2">
         <v>7.6</v>
       </c>
       <c r="J177">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K177" s="1">
-        <v>7.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:11">
@@ -25034,25 +25034,25 @@
         <v>226</v>
       </c>
       <c r="E183">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F183">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G183" s="1">
-        <v>95.09999999999999</v>
+        <v>96</v>
       </c>
       <c r="H183" s="1">
-        <v>4.9</v>
+        <v>4</v>
       </c>
       <c r="I183" s="2">
         <v>7.6</v>
       </c>
       <c r="J183">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>1.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -25483,25 +25483,25 @@
         <v>42</v>
       </c>
       <c r="E196">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F196">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G196" s="1">
-        <v>66.7</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H196" s="1">
-        <v>33.3</v>
+        <v>7.1</v>
       </c>
       <c r="I196" s="2">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="J196">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="K196" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197" spans="1:11">
@@ -25518,25 +25518,25 @@
         <v>36</v>
       </c>
       <c r="E197">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F197">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G197" s="1">
-        <v>88.90000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="H197" s="1">
-        <v>11.1</v>
+        <v>2.8</v>
       </c>
       <c r="I197" s="2">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="J197">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K197" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:11">
@@ -25553,25 +25553,25 @@
         <v>36</v>
       </c>
       <c r="E198">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F198">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G198" s="1">
-        <v>91.7</v>
+        <v>97.2</v>
       </c>
       <c r="H198" s="1">
-        <v>8.300000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="I198" s="2">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="J198">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K198" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:11">
@@ -25585,25 +25585,25 @@
         <v>114</v>
       </c>
       <c r="E199">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="F199">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="G199" s="1">
-        <v>81.59999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="H199" s="1">
-        <v>18.4</v>
+        <v>4.4</v>
       </c>
       <c r="I199" s="2">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="J199">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="K199" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:11">
@@ -26923,25 +26923,25 @@
         <v>32</v>
       </c>
       <c r="E238">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F238">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G238" s="1">
-        <v>78.09999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="H238" s="1">
-        <v>21.9</v>
+        <v>18.8</v>
       </c>
       <c r="I238" s="2">
         <v>6.8</v>
       </c>
       <c r="J238">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="K238" s="1">
-        <v>100</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="239" spans="1:11">
@@ -27130,25 +27130,25 @@
         <v>172</v>
       </c>
       <c r="E244">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F244">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G244" s="1">
-        <v>95.90000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="H244" s="1">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="I244" s="2">
         <v>7.4</v>
       </c>
       <c r="J244">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="K244" s="1">
-        <v>18.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="245" spans="1:11">
@@ -27442,25 +27442,25 @@
         <v>33</v>
       </c>
       <c r="E253">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F253">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G253" s="1">
-        <v>60.6</v>
+        <v>81.8</v>
       </c>
       <c r="H253" s="1">
-        <v>39.4</v>
+        <v>18.2</v>
       </c>
       <c r="I253" s="2">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="J253">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K253" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254" spans="1:11">
@@ -27474,25 +27474,25 @@
         <v>103</v>
       </c>
       <c r="E254">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F254">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G254" s="1">
-        <v>68</v>
+        <v>74.8</v>
       </c>
       <c r="H254" s="1">
-        <v>32</v>
+        <v>25.2</v>
       </c>
       <c r="I254" s="2">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="J254">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K254" s="1">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="255" spans="1:11">

</xml_diff>